<commit_message>
vault backup: 2026-10-13 20:55:37
</commit_message>
<xml_diff>
--- a/Dashboards/Areas/💰 Finance/Household Budget 2026-10.xlsx
+++ b/Dashboards/Areas/💰 Finance/Household Budget 2026-10.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="473">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="478">
   <si>
     <t xml:space="preserve">Household Budget — October 2026 rebuild</t>
   </si>
@@ -772,7 +772,22 @@
     <t xml:space="preserve">Pre-funds camp/trips due before enough has built up (Sinking Funds sheet). Your stack: debt → liquidity → lifestyle → investible. Overwrite to change.</t>
   </si>
   <si>
-    <t xml:space="preserve">Diogo base salary</t>
+    <t xml:space="preserve">Flagship base salary (bonus basis)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per you: the March bonus is paid on the current $339k.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New base salary (from 11/2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per you. The March raise applies to this.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net effect of the +$1k base from Nov-26 (per month)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(New − old salary) × net share ÷ 12. Take-home otherwise assumed unchanged.</t>
   </si>
   <si>
     <t xml:space="preserve">Cost-of-living raise %</t>
@@ -1441,7 +1456,7 @@
     <t xml:space="preserve">Categories are keyword-based on merchant strings; unclassified items are shown on Actuals. Weekly checks = cleaning help ($160/wk); DoorDash/Grubhub = family takeout (per you). HELOC payment of ~$1,100 is assumed from Nov-26. Synchrony = 0% AC-repair loan; Wells Fargo = 0% plumbing loan, assumed $450/mo (one payment seen).</t>
   </si>
   <si>
-    <t xml:space="preserve">Job change: new job starts 11/2. Take-home is assumed unchanged at the new employer (pay, cadence and benefits not yet known). Bonus = 25% of $339k at an assumed 1.00 multiplier, paid in March net of withholding; ~$4k extra tax is reserved for April. Raise (3% midpoint of your 2–4%) starts in March with 2 months of back pay (assumed Jan 1).</t>
+    <t xml:space="preserve">Job change: new job starts 11/2. Pay cadence is unchanged and the first new-employer paycheck is 11/15 (no missed paycheck); take-home is assumed unchanged apart from +$50/mo from the $1k higher base. Benefits start date still unknown. Bonus = 25% of $339k at an assumed 1.00 multiplier, paid in March net of withholding; ~$4k extra tax is reserved for April. Raise (3% midpoint of your 2–4%) applies to the new $340k base, starts in March, with 2 months of back pay (assumed Jan 1).</t>
   </si>
   <si>
     <t xml:space="preserve">Not financial, tax, or legal advice.</t>
@@ -4616,7 +4631,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:W90"/>
+  <dimension ref="A1:W92"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
@@ -4670,7 +4685,7 @@
         <v>195</v>
       </c>
       <c r="G5" s="29" t="n">
-        <f aca="false">IFERROR(INDEX(A43:A90,MATCH(1,Q43:Q90,0)),"after Oct-30")</f>
+        <f aca="false">IFERROR(INDEX(A45:A92,MATCH(1,Q45:Q92,0)),"after Oct-30")</f>
         <v>46447</v>
       </c>
     </row>
@@ -4688,7 +4703,7 @@
         <v>198</v>
       </c>
       <c r="G6" s="29" t="n">
-        <f aca="false">IFERROR(INDEX(A43:A90,MATCH(1,R43:R90,0)),"after Oct-30")</f>
+        <f aca="false">IFERROR(INDEX(A45:A92,MATCH(1,R45:R92,0)),"after Oct-30")</f>
         <v>46447</v>
       </c>
     </row>
@@ -4706,7 +4721,7 @@
         <v>200</v>
       </c>
       <c r="G7" s="29" t="n">
-        <f aca="false">IFERROR(INDEX(A43:A90,MATCH(1,S43:S90,0)),"after Oct-30")</f>
+        <f aca="false">IFERROR(INDEX(A45:A92,MATCH(1,S45:S92,0)),"after Oct-30")</f>
         <v>46447</v>
       </c>
     </row>
@@ -4724,7 +4739,7 @@
         <v>202</v>
       </c>
       <c r="G8" s="29" t="n">
-        <f aca="false">IFERROR(INDEX(A43:A90,MATCH(1,T43:T90,0)),"after Oct-30")</f>
+        <f aca="false">IFERROR(INDEX(A45:A92,MATCH(1,T45:T92,0)),"after Oct-30")</f>
         <v>46447</v>
       </c>
     </row>
@@ -4742,8 +4757,8 @@
         <v>205</v>
       </c>
       <c r="G9" s="29" t="n">
-        <f aca="false">IFERROR(INDEX(A43:A90,MATCH(1,U43:U90,0)),"after Oct-30")</f>
-        <v>46905</v>
+        <f aca="false">IFERROR(INDEX(A45:A92,MATCH(1,U45:U92,0)),"after Oct-30")</f>
+        <v>46874</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4760,8 +4775,8 @@
         <v>208</v>
       </c>
       <c r="G10" s="9" t="n">
-        <f aca="false">SUM(F43:F90)+SUM(J43:J90)</f>
-        <v>1455.31534406423</v>
+        <f aca="false">SUM(F45:F92)+SUM(J45:J92)</f>
+        <v>1442.47513468667</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5000,419 +5015,256 @@
         <v>339000</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>233</v>
+        <v>249</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>249</v>
-      </c>
-      <c r="B31" s="33" t="n">
-        <v>0.03</v>
+        <v>250</v>
+      </c>
+      <c r="B31" s="13" t="n">
+        <v>340000</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>251</v>
-      </c>
-      <c r="B32" s="33" t="n">
-        <v>0.6065</v>
+        <v>252</v>
+      </c>
+      <c r="B32" s="12" t="n">
+        <f aca="false">($B$31-$B$30)*$B$34/12</f>
+        <v>50.5416666666667</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="B33" s="26" t="n">
-        <v>46447</v>
+        <v>254</v>
+      </c>
+      <c r="B33" s="33" t="n">
+        <v>0.03</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="B34" s="7" t="n">
-        <v>2</v>
+        <v>256</v>
+      </c>
+      <c r="B34" s="33" t="n">
+        <v>0.6065</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="B35" s="12" t="n">
-        <f aca="false">$B$30*$B$31*$B$32/12</f>
-        <v>514.00875</v>
+        <v>258</v>
+      </c>
+      <c r="B35" s="26" t="n">
+        <v>46447</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>259</v>
-      </c>
-      <c r="B36" s="13" t="n">
-        <v>0</v>
+        <v>260</v>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>2</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>261</v>
-      </c>
-      <c r="B37" s="26" t="n">
-        <v>46447</v>
-      </c>
-      <c r="C37" s="2"/>
+        <v>262</v>
+      </c>
+      <c r="B37" s="12" t="n">
+        <f aca="false">$B$31*$B$33*$B$34/12</f>
+        <v>515.525</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>263</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>262</v>
-      </c>
-      <c r="B38" s="26" t="n">
-        <v>47119</v>
+        <v>264</v>
+      </c>
+      <c r="B38" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>264</v>
-      </c>
-      <c r="B39" s="21" t="n">
+        <v>266</v>
+      </c>
+      <c r="B39" s="26" t="n">
+        <v>46447</v>
+      </c>
+      <c r="C39" s="2"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="B40" s="26" t="n">
+        <v>47119</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="B41" s="21" t="n">
         <f aca="false">Budget!F16</f>
         <v>342</v>
       </c>
-      <c r="C39" s="2" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="10" t="s">
-        <v>266</v>
-      </c>
-      <c r="B42" s="10" t="s">
-        <v>267</v>
-      </c>
-      <c r="C42" s="10" t="s">
-        <v>268</v>
-      </c>
-      <c r="D42" s="10" t="s">
-        <v>269</v>
-      </c>
-      <c r="E42" s="10" t="s">
+      <c r="C41" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="F42" s="10" t="s">
+    </row>
+    <row r="44" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="10" t="s">
         <v>271</v>
       </c>
-      <c r="G42" s="10" t="s">
+      <c r="B44" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="H42" s="10" t="s">
+      <c r="C44" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="I42" s="10" t="s">
+      <c r="D44" s="10" t="s">
         <v>274</v>
       </c>
-      <c r="J42" s="10" t="s">
+      <c r="E44" s="10" t="s">
         <v>275</v>
       </c>
-      <c r="K42" s="10" t="s">
+      <c r="F44" s="10" t="s">
         <v>276</v>
       </c>
-      <c r="L42" s="10" t="s">
+      <c r="G44" s="10" t="s">
         <v>277</v>
       </c>
-      <c r="M42" s="10" t="s">
+      <c r="H44" s="10" t="s">
         <v>278</v>
       </c>
-      <c r="N42" s="10" t="s">
+      <c r="I44" s="10" t="s">
         <v>279</v>
       </c>
-      <c r="O42" s="10" t="s">
+      <c r="J44" s="10" t="s">
         <v>280</v>
       </c>
-      <c r="P42" s="10" t="s">
+      <c r="K44" s="10" t="s">
         <v>281</v>
       </c>
-      <c r="Q42" s="10" t="s">
+      <c r="L44" s="10" t="s">
         <v>282</v>
       </c>
-      <c r="R42" s="10" t="s">
+      <c r="M44" s="10" t="s">
         <v>283</v>
       </c>
-      <c r="S42" s="10" t="s">
+      <c r="N44" s="10" t="s">
         <v>284</v>
       </c>
-      <c r="T42" s="10" t="s">
+      <c r="O44" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="U42" s="10" t="s">
+      <c r="P44" s="10" t="s">
         <v>286</v>
       </c>
-      <c r="V42" s="10" t="s">
+      <c r="Q44" s="10" t="s">
         <v>287</v>
       </c>
-      <c r="W42" s="10" t="s">
+      <c r="R44" s="10" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="34" t="n">
+      <c r="S44" s="10" t="s">
+        <v>289</v>
+      </c>
+      <c r="T44" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="U44" s="10" t="s">
+        <v>291</v>
+      </c>
+      <c r="V44" s="10" t="s">
+        <v>292</v>
+      </c>
+      <c r="W44" s="10" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="34" t="n">
         <v>46327</v>
       </c>
-      <c r="B43" s="21" t="n">
-        <f aca="false">IF(A43&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A43&gt;$B$38,$B$39,0)+IF(A43&gt;=$B$33,$B$35,0)</f>
-        <v>926.776666666669</v>
-      </c>
-      <c r="C43" s="12" t="n">
-        <f aca="false">IF(A43=$B$37,$B$26-$B$29,0)-IF(A43=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A43=$B$33,$B$35*$B$34,0)+$B$36</f>
-        <v>0</v>
-      </c>
-      <c r="D43" s="12" t="n">
-        <f aca="false">B43+C43</f>
-        <v>926.776666666669</v>
-      </c>
-      <c r="E43" s="12" t="n">
+      <c r="B45" s="21" t="n">
+        <f aca="false">IF(A45&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A45&gt;$B$40,$B$41,0)+IF(A45&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>977.318333333335</v>
+      </c>
+      <c r="C45" s="12" t="n">
+        <f aca="false">IF(A45=$B$39,$B$26-$B$29,0)-IF(A45=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A45=$B$35,$B$37*$B$36,0)+$B$38</f>
+        <v>0</v>
+      </c>
+      <c r="D45" s="12" t="n">
+        <f aca="false">B45+C45</f>
+        <v>977.318333333335</v>
+      </c>
+      <c r="E45" s="12" t="n">
         <f aca="false">$B$5</f>
         <v>9800.78</v>
       </c>
-      <c r="F43" s="12" t="n">
-        <f aca="false">E43*$B$6/12</f>
+      <c r="F45" s="12" t="n">
+        <f aca="false">E45*$B$6/12</f>
         <v>242.895997666667</v>
       </c>
-      <c r="G43" s="12" t="n">
-        <f aca="false">MIN(E43+F43,MAX(D43-K43,0))</f>
-        <v>795.508812666668</v>
-      </c>
-      <c r="H43" s="12" t="n">
-        <f aca="false">E43+F43-G43</f>
-        <v>9248.167185</v>
-      </c>
-      <c r="I43" s="12" t="n">
+      <c r="G45" s="12" t="n">
+        <f aca="false">MIN(E45+F45,MAX(D45-K45,0))</f>
+        <v>846.050479333335</v>
+      </c>
+      <c r="H45" s="12" t="n">
+        <f aca="false">E45+F45-G45</f>
+        <v>9197.62551833333</v>
+      </c>
+      <c r="I45" s="12" t="n">
         <f aca="false">$B$7</f>
         <v>5341.52</v>
       </c>
-      <c r="J43" s="12" t="n">
-        <f aca="false">I43*$B$8/12</f>
-        <v>77.852654</v>
-      </c>
-      <c r="K43" s="12" t="n">
-        <f aca="false">MIN(I43+J43,J43+$B$9*I43)</f>
-        <v>131.267854</v>
-      </c>
-      <c r="L43" s="12" t="n">
-        <f aca="false">MIN(I43+J43,MAX(D43-G43,0))</f>
-        <v>131.267854</v>
-      </c>
-      <c r="M43" s="12" t="n">
-        <f aca="false">I43+J43-L43</f>
-        <v>5288.1048</v>
-      </c>
-      <c r="N43" s="12" t="n">
-        <f aca="false">$B$10-$B$36</f>
-        <v>12081</v>
-      </c>
-      <c r="O43" s="12" t="n">
-        <f aca="false">MIN(D43-G43-L43,MAX($B$15-$B$18-N43,0))</f>
-        <v>0</v>
-      </c>
-      <c r="P43" s="12" t="n">
-        <f aca="false">N43+O43</f>
-        <v>12081</v>
-      </c>
-      <c r="Q43" s="5" t="n">
-        <f aca="false">IF(H43&lt;=0.005,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="R43" s="5" t="n">
-        <f aca="false">IF(M43&lt;=0.005,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="S43" s="5" t="n">
-        <f aca="false">IF(AND(Q43=1,R43=1),1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="T43" s="5" t="n">
-        <f aca="false">IF(P43&gt;=$B$20,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="U43" s="5" t="n">
-        <f aca="false">IF(P43+$B$18&gt;=$B$15-0.5,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="V43" s="12" t="n">
-        <f aca="false">MAX(D43-G43-L43,0)-MAX(O43,0)</f>
-        <v>0</v>
-      </c>
-      <c r="W43" s="12" t="n">
-        <f aca="false">P43+$B$18</f>
-        <v>28341.75</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="34" t="n">
-        <v>46357</v>
-      </c>
-      <c r="B44" s="21" t="n">
-        <f aca="false">IF(A44&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A44&gt;$B$38,$B$39,0)+IF(A44&gt;=$B$33,$B$35,0)</f>
-        <v>926.776666666669</v>
-      </c>
-      <c r="C44" s="12" t="n">
-        <f aca="false">IF(A44=$B$37,$B$26-$B$29,0)-IF(A44=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A44=$B$33,$B$35*$B$34,0)+0</f>
-        <v>0</v>
-      </c>
-      <c r="D44" s="12" t="n">
-        <f aca="false">B44+C44</f>
-        <v>926.776666666669</v>
-      </c>
-      <c r="E44" s="12" t="n">
-        <f aca="false">H43</f>
-        <v>9248.167185</v>
-      </c>
-      <c r="F44" s="12" t="n">
-        <f aca="false">E44*$B$6/12</f>
-        <v>229.20041006825</v>
-      </c>
-      <c r="G44" s="12" t="n">
-        <f aca="false">MIN(E44+F44,MAX(D44-K44,0))</f>
-        <v>796.821491206669</v>
-      </c>
-      <c r="H44" s="12" t="n">
-        <f aca="false">E44+F44-G44</f>
-        <v>8680.54610386158</v>
-      </c>
-      <c r="I44" s="12" t="n">
-        <f aca="false">M43</f>
-        <v>5288.1048</v>
-      </c>
-      <c r="J44" s="12" t="n">
-        <f aca="false">I44*$B$8/12</f>
-        <v>77.07412746</v>
-      </c>
-      <c r="K44" s="12" t="n">
-        <f aca="false">MIN(I44+J44,J44+$B$9*I44)</f>
-        <v>129.95517546</v>
-      </c>
-      <c r="L44" s="12" t="n">
-        <f aca="false">MIN(I44+J44,MAX(D44-G44,0))</f>
-        <v>129.95517546</v>
-      </c>
-      <c r="M44" s="12" t="n">
-        <f aca="false">I44+J44-L44</f>
-        <v>5235.223752</v>
-      </c>
-      <c r="N44" s="12" t="n">
-        <f aca="false">P43</f>
-        <v>12081</v>
-      </c>
-      <c r="O44" s="12" t="n">
-        <f aca="false">MIN(D44-G44-L44,MAX($B$15-$B$18-N44,0))</f>
-        <v>0</v>
-      </c>
-      <c r="P44" s="12" t="n">
-        <f aca="false">N44+O44</f>
-        <v>12081</v>
-      </c>
-      <c r="Q44" s="5" t="n">
-        <f aca="false">IF(H44&lt;=0.005,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="R44" s="5" t="n">
-        <f aca="false">IF(M44&lt;=0.005,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="S44" s="5" t="n">
-        <f aca="false">IF(AND(Q44=1,R44=1),1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="T44" s="5" t="n">
-        <f aca="false">IF(P44&gt;=$B$20,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="U44" s="5" t="n">
-        <f aca="false">IF(P44+$B$18&gt;=$B$15-0.5,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="V44" s="12" t="n">
-        <f aca="false">MAX(D44-G44-L44,0)-MAX(O44,0)</f>
-        <v>0</v>
-      </c>
-      <c r="W44" s="12" t="n">
-        <f aca="false">P44+$B$18</f>
-        <v>28341.75</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="34" t="n">
-        <v>46388</v>
-      </c>
-      <c r="B45" s="21" t="n">
-        <f aca="false">IF(A45&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A45&gt;$B$38,$B$39,0)+IF(A45&gt;=$B$33,$B$35,0)</f>
-        <v>926.776666666669</v>
-      </c>
-      <c r="C45" s="12" t="n">
-        <f aca="false">IF(A45=$B$37,$B$26-$B$29,0)-IF(A45=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A45=$B$33,$B$35*$B$34,0)+0</f>
-        <v>0</v>
-      </c>
-      <c r="D45" s="12" t="n">
-        <f aca="false">B45+C45</f>
-        <v>926.776666666669</v>
-      </c>
-      <c r="E45" s="12" t="n">
-        <f aca="false">H44</f>
-        <v>8680.54610386158</v>
-      </c>
-      <c r="F45" s="12" t="n">
-        <f aca="false">E45*$B$6/12</f>
-        <v>215.132867607369</v>
-      </c>
-      <c r="G45" s="12" t="n">
-        <f aca="false">MIN(E45+F45,MAX(D45-K45,0))</f>
-        <v>798.121042961268</v>
-      </c>
-      <c r="H45" s="12" t="n">
-        <f aca="false">E45+F45-G45</f>
-        <v>8097.55792850768</v>
-      </c>
-      <c r="I45" s="12" t="n">
-        <f aca="false">M44</f>
-        <v>5235.223752</v>
-      </c>
       <c r="J45" s="12" t="n">
         <f aca="false">I45*$B$8/12</f>
-        <v>76.3033861854</v>
+        <v>77.852654</v>
       </c>
       <c r="K45" s="12" t="n">
         <f aca="false">MIN(I45+J45,J45+$B$9*I45)</f>
-        <v>128.6556237054</v>
+        <v>131.267854</v>
       </c>
       <c r="L45" s="12" t="n">
         <f aca="false">MIN(I45+J45,MAX(D45-G45,0))</f>
-        <v>128.6556237054</v>
+        <v>131.267854</v>
       </c>
       <c r="M45" s="12" t="n">
         <f aca="false">I45+J45-L45</f>
-        <v>5182.87151448</v>
+        <v>5288.1048</v>
       </c>
       <c r="N45" s="12" t="n">
-        <f aca="false">P44</f>
+        <f aca="false">$B$10-$B$38</f>
         <v>12081</v>
       </c>
       <c r="O45" s="12" t="n">
@@ -5454,55 +5306,55 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="34" t="n">
-        <v>46419</v>
+        <v>46357</v>
       </c>
       <c r="B46" s="21" t="n">
-        <f aca="false">IF(A46&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A46&gt;$B$38,$B$39,0)+IF(A46&gt;=$B$33,$B$35,0)</f>
-        <v>926.776666666669</v>
+        <f aca="false">IF(A46&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A46&gt;$B$40,$B$41,0)+IF(A46&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>977.318333333335</v>
       </c>
       <c r="C46" s="12" t="n">
-        <f aca="false">IF(A46=$B$37,$B$26-$B$29,0)-IF(A46=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A46=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A46=$B$39,$B$26-$B$29,0)-IF(A46=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A46=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D46" s="12" t="n">
         <f aca="false">B46+C46</f>
-        <v>926.776666666669</v>
+        <v>977.318333333335</v>
       </c>
       <c r="E46" s="12" t="n">
         <f aca="false">H45</f>
-        <v>8097.55792850768</v>
+        <v>9197.62551833333</v>
       </c>
       <c r="F46" s="12" t="n">
         <f aca="false">E46*$B$6/12</f>
-        <v>200.684477328182</v>
+        <v>227.947819096028</v>
       </c>
       <c r="G46" s="12" t="n">
         <f aca="false">MIN(E46+F46,MAX(D46-K46,0))</f>
-        <v>799.407599198322</v>
+        <v>847.363157873335</v>
       </c>
       <c r="H46" s="12" t="n">
         <f aca="false">E46+F46-G46</f>
-        <v>7498.83480663754</v>
+        <v>8578.21017955603</v>
       </c>
       <c r="I46" s="12" t="n">
         <f aca="false">M45</f>
-        <v>5182.87151448</v>
+        <v>5288.1048</v>
       </c>
       <c r="J46" s="12" t="n">
         <f aca="false">I46*$B$8/12</f>
-        <v>75.540352323546</v>
+        <v>77.07412746</v>
       </c>
       <c r="K46" s="12" t="n">
         <f aca="false">MIN(I46+J46,J46+$B$9*I46)</f>
-        <v>127.369067468346</v>
+        <v>129.95517546</v>
       </c>
       <c r="L46" s="12" t="n">
         <f aca="false">MIN(I46+J46,MAX(D46-G46,0))</f>
-        <v>127.369067468346</v>
+        <v>129.95517546</v>
       </c>
       <c r="M46" s="12" t="n">
         <f aca="false">I46+J46-L46</f>
-        <v>5131.0427993352</v>
+        <v>5235.223752</v>
       </c>
       <c r="N46" s="12" t="n">
         <f aca="false">P45</f>
@@ -5547,55 +5399,55 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="34" t="n">
-        <v>46447</v>
+        <v>46388</v>
       </c>
       <c r="B47" s="21" t="n">
-        <f aca="false">IF(A47&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A47&gt;$B$38,$B$39,0)+IF(A47&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A47&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A47&gt;$B$40,$B$41,0)+IF(A47&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>977.318333333335</v>
       </c>
       <c r="C47" s="12" t="n">
-        <f aca="false">IF(A47=$B$37,$B$26-$B$29,0)-IF(A47=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A47=$B$33,$B$35*$B$34,0)+0</f>
-        <v>51578.8091666667</v>
+        <f aca="false">IF(A47=$B$39,$B$26-$B$29,0)-IF(A47=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A47=$B$35,$B$37*$B$36,0)+0</f>
+        <v>0</v>
       </c>
       <c r="D47" s="12" t="n">
         <f aca="false">B47+C47</f>
-        <v>54095.8445833333</v>
+        <v>977.318333333335</v>
       </c>
       <c r="E47" s="12" t="n">
         <f aca="false">H46</f>
-        <v>7498.83480663754</v>
+        <v>8578.21017955603</v>
       </c>
       <c r="F47" s="12" t="n">
         <f aca="false">E47*$B$6/12</f>
-        <v>185.8461226245</v>
+        <v>212.59664228333</v>
       </c>
       <c r="G47" s="12" t="n">
         <f aca="false">MIN(E47+F47,MAX(D47-K47,0))</f>
-        <v>7684.68092926204</v>
+        <v>848.662709627935</v>
       </c>
       <c r="H47" s="12" t="n">
         <f aca="false">E47+F47-G47</f>
-        <v>0</v>
+        <v>7942.14411221142</v>
       </c>
       <c r="I47" s="12" t="n">
         <f aca="false">M46</f>
-        <v>5131.0427993352</v>
+        <v>5235.223752</v>
       </c>
       <c r="J47" s="12" t="n">
         <f aca="false">I47*$B$8/12</f>
-        <v>74.7849488003106</v>
+        <v>76.3033861854</v>
       </c>
       <c r="K47" s="12" t="n">
         <f aca="false">MIN(I47+J47,J47+$B$9*I47)</f>
-        <v>126.095376793663</v>
+        <v>128.6556237054</v>
       </c>
       <c r="L47" s="12" t="n">
         <f aca="false">MIN(I47+J47,MAX(D47-G47,0))</f>
-        <v>5205.82774813551</v>
+        <v>128.6556237054</v>
       </c>
       <c r="M47" s="12" t="n">
         <f aca="false">I47+J47-L47</f>
-        <v>0</v>
+        <v>5182.87151448</v>
       </c>
       <c r="N47" s="12" t="n">
         <f aca="false">P46</f>
@@ -5603,27 +5455,27 @@
       </c>
       <c r="O47" s="12" t="n">
         <f aca="false">MIN(D47-G47-L47,MAX($B$15-$B$18-N47,0))</f>
-        <v>41205.3359059358</v>
+        <v>0</v>
       </c>
       <c r="P47" s="12" t="n">
         <f aca="false">N47+O47</f>
-        <v>53286.3359059358</v>
+        <v>12081</v>
       </c>
       <c r="Q47" s="5" t="n">
         <f aca="false">IF(H47&lt;=0.005,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R47" s="5" t="n">
         <f aca="false">IF(M47&lt;=0.005,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S47" s="5" t="n">
         <f aca="false">IF(AND(Q47=1,R47=1),1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T47" s="5" t="n">
         <f aca="false">IF(P47&gt;=$B$20,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U47" s="5" t="n">
         <f aca="false">IF(P47+$B$18&gt;=$B$15-0.5,1,0)</f>
@@ -5635,88 +5487,88 @@
       </c>
       <c r="W47" s="12" t="n">
         <f aca="false">P47+$B$18</f>
-        <v>69547.0859059358</v>
+        <v>28341.75</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="34" t="n">
-        <v>46478</v>
+        <v>46419</v>
       </c>
       <c r="B48" s="21" t="n">
-        <f aca="false">IF(A48&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A48&gt;$B$38,$B$39,0)+IF(A48&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A48&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A48&gt;$B$40,$B$41,0)+IF(A48&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>977.318333333335</v>
       </c>
       <c r="C48" s="12" t="n">
-        <f aca="false">IF(A48=$B$37,$B$26-$B$29,0)-IF(A48=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A48=$B$33,$B$35*$B$34,0)+0</f>
-        <v>-3983.25</v>
+        <f aca="false">IF(A48=$B$39,$B$26-$B$29,0)-IF(A48=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A48=$B$35,$B$37*$B$36,0)+0</f>
+        <v>0</v>
       </c>
       <c r="D48" s="12" t="n">
         <f aca="false">B48+C48</f>
-        <v>-1466.21458333333</v>
+        <v>977.318333333335</v>
       </c>
       <c r="E48" s="12" t="n">
         <f aca="false">H47</f>
-        <v>0</v>
+        <v>7942.14411221142</v>
       </c>
       <c r="F48" s="12" t="n">
         <f aca="false">E48*$B$6/12</f>
-        <v>0</v>
+        <v>196.832804914306</v>
       </c>
       <c r="G48" s="12" t="n">
         <f aca="false">MIN(E48+F48,MAX(D48-K48,0))</f>
-        <v>0</v>
+        <v>849.949265864989</v>
       </c>
       <c r="H48" s="12" t="n">
         <f aca="false">E48+F48-G48</f>
-        <v>0</v>
+        <v>7289.02765126074</v>
       </c>
       <c r="I48" s="12" t="n">
         <f aca="false">M47</f>
-        <v>0</v>
+        <v>5182.87151448</v>
       </c>
       <c r="J48" s="12" t="n">
         <f aca="false">I48*$B$8/12</f>
-        <v>0</v>
+        <v>75.540352323546</v>
       </c>
       <c r="K48" s="12" t="n">
         <f aca="false">MIN(I48+J48,J48+$B$9*I48)</f>
-        <v>0</v>
+        <v>127.369067468346</v>
       </c>
       <c r="L48" s="12" t="n">
         <f aca="false">MIN(I48+J48,MAX(D48-G48,0))</f>
-        <v>0</v>
+        <v>127.369067468346</v>
       </c>
       <c r="M48" s="12" t="n">
         <f aca="false">I48+J48-L48</f>
-        <v>0</v>
+        <v>5131.0427993352</v>
       </c>
       <c r="N48" s="12" t="n">
         <f aca="false">P47</f>
-        <v>53286.3359059358</v>
+        <v>12081</v>
       </c>
       <c r="O48" s="12" t="n">
         <f aca="false">MIN(D48-G48-L48,MAX($B$15-$B$18-N48,0))</f>
-        <v>-1466.21458333333</v>
+        <v>0</v>
       </c>
       <c r="P48" s="12" t="n">
         <f aca="false">N48+O48</f>
-        <v>51820.1213226025</v>
+        <v>12081</v>
       </c>
       <c r="Q48" s="5" t="n">
         <f aca="false">IF(H48&lt;=0.005,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R48" s="5" t="n">
         <f aca="false">IF(M48&lt;=0.005,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S48" s="5" t="n">
         <f aca="false">IF(AND(Q48=1,R48=1),1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T48" s="5" t="n">
         <f aca="false">IF(P48&gt;=$B$20,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U48" s="5" t="n">
         <f aca="false">IF(P48+$B$18&gt;=$B$15-0.5,1,0)</f>
@@ -5728,36 +5580,36 @@
       </c>
       <c r="W48" s="12" t="n">
         <f aca="false">P48+$B$18</f>
-        <v>68080.8713226024</v>
+        <v>28341.75</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="34" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="B49" s="21" t="n">
-        <f aca="false">IF(A49&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A49&gt;$B$38,$B$39,0)+IF(A49&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A49&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A49&gt;$B$40,$B$41,0)+IF(A49&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C49" s="12" t="n">
-        <f aca="false">IF(A49=$B$37,$B$26-$B$29,0)-IF(A49=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A49=$B$33,$B$35*$B$34,0)+0</f>
-        <v>0</v>
+        <f aca="false">IF(A49=$B$39,$B$26-$B$29,0)-IF(A49=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A49=$B$35,$B$37*$B$36,0)+0</f>
+        <v>51581.8416666667</v>
       </c>
       <c r="D49" s="12" t="n">
         <f aca="false">B49+C49</f>
-        <v>2517.03541666667</v>
+        <v>54150.935</v>
       </c>
       <c r="E49" s="12" t="n">
         <f aca="false">H48</f>
-        <v>0</v>
+        <v>7289.02765126074</v>
       </c>
       <c r="F49" s="12" t="n">
         <f aca="false">E49*$B$6/12</f>
-        <v>0</v>
+        <v>180.646401957079</v>
       </c>
       <c r="G49" s="12" t="n">
         <f aca="false">MIN(E49+F49,MAX(D49-K49,0))</f>
-        <v>0</v>
+        <v>7469.67405321782</v>
       </c>
       <c r="H49" s="12" t="n">
         <f aca="false">E49+F49-G49</f>
@@ -5765,19 +5617,19 @@
       </c>
       <c r="I49" s="12" t="n">
         <f aca="false">M48</f>
-        <v>0</v>
+        <v>5131.0427993352</v>
       </c>
       <c r="J49" s="12" t="n">
         <f aca="false">I49*$B$8/12</f>
-        <v>0</v>
+        <v>74.7849488003106</v>
       </c>
       <c r="K49" s="12" t="n">
         <f aca="false">MIN(I49+J49,J49+$B$9*I49)</f>
-        <v>0</v>
+        <v>126.095376793663</v>
       </c>
       <c r="L49" s="12" t="n">
         <f aca="false">MIN(I49+J49,MAX(D49-G49,0))</f>
-        <v>0</v>
+        <v>5205.82774813551</v>
       </c>
       <c r="M49" s="12" t="n">
         <f aca="false">I49+J49-L49</f>
@@ -5785,15 +5637,15 @@
       </c>
       <c r="N49" s="12" t="n">
         <f aca="false">P48</f>
-        <v>51820.1213226025</v>
+        <v>12081</v>
       </c>
       <c r="O49" s="12" t="n">
         <f aca="false">MIN(D49-G49-L49,MAX($B$15-$B$18-N49,0))</f>
-        <v>2517.03541666667</v>
+        <v>41475.4331986467</v>
       </c>
       <c r="P49" s="12" t="n">
         <f aca="false">N49+O49</f>
-        <v>54337.1567392691</v>
+        <v>53556.4331986467</v>
       </c>
       <c r="Q49" s="5" t="n">
         <f aca="false">IF(H49&lt;=0.005,1,0)</f>
@@ -5821,24 +5673,24 @@
       </c>
       <c r="W49" s="12" t="n">
         <f aca="false">P49+$B$18</f>
-        <v>70597.9067392691</v>
+        <v>69817.1831986467</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="34" t="n">
-        <v>46539</v>
+        <v>46478</v>
       </c>
       <c r="B50" s="21" t="n">
-        <f aca="false">IF(A50&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A50&gt;$B$38,$B$39,0)+IF(A50&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A50&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A50&gt;$B$40,$B$41,0)+IF(A50&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C50" s="12" t="n">
-        <f aca="false">IF(A50=$B$37,$B$26-$B$29,0)-IF(A50=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A50=$B$33,$B$35*$B$34,0)+0</f>
-        <v>0</v>
+        <f aca="false">IF(A50=$B$39,$B$26-$B$29,0)-IF(A50=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A50=$B$35,$B$37*$B$36,0)+0</f>
+        <v>-3983.25</v>
       </c>
       <c r="D50" s="12" t="n">
         <f aca="false">B50+C50</f>
-        <v>2517.03541666667</v>
+        <v>-1414.15666666667</v>
       </c>
       <c r="E50" s="12" t="n">
         <f aca="false">H49</f>
@@ -5878,15 +5730,15 @@
       </c>
       <c r="N50" s="12" t="n">
         <f aca="false">P49</f>
-        <v>54337.1567392691</v>
+        <v>53556.4331986467</v>
       </c>
       <c r="O50" s="12" t="n">
         <f aca="false">MIN(D50-G50-L50,MAX($B$15-$B$18-N50,0))</f>
-        <v>2517.03541666667</v>
+        <v>-1414.15666666667</v>
       </c>
       <c r="P50" s="12" t="n">
         <f aca="false">N50+O50</f>
-        <v>56854.1921559358</v>
+        <v>52142.27653198</v>
       </c>
       <c r="Q50" s="5" t="n">
         <f aca="false">IF(H50&lt;=0.005,1,0)</f>
@@ -5914,24 +5766,24 @@
       </c>
       <c r="W50" s="12" t="n">
         <f aca="false">P50+$B$18</f>
-        <v>73114.9421559358</v>
+        <v>68403.02653198</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="34" t="n">
-        <v>46569</v>
+        <v>46508</v>
       </c>
       <c r="B51" s="21" t="n">
-        <f aca="false">IF(A51&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A51&gt;$B$38,$B$39,0)+IF(A51&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A51&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A51&gt;$B$40,$B$41,0)+IF(A51&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C51" s="12" t="n">
-        <f aca="false">IF(A51=$B$37,$B$26-$B$29,0)-IF(A51=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A51=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A51=$B$39,$B$26-$B$29,0)-IF(A51=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A51=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D51" s="12" t="n">
         <f aca="false">B51+C51</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E51" s="12" t="n">
         <f aca="false">H50</f>
@@ -5971,15 +5823,15 @@
       </c>
       <c r="N51" s="12" t="n">
         <f aca="false">P50</f>
-        <v>56854.1921559358</v>
+        <v>52142.27653198</v>
       </c>
       <c r="O51" s="12" t="n">
         <f aca="false">MIN(D51-G51-L51,MAX($B$15-$B$18-N51,0))</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="P51" s="12" t="n">
         <f aca="false">N51+O51</f>
-        <v>59371.2275726024</v>
+        <v>54711.3698653134</v>
       </c>
       <c r="Q51" s="5" t="n">
         <f aca="false">IF(H51&lt;=0.005,1,0)</f>
@@ -6007,24 +5859,24 @@
       </c>
       <c r="W51" s="12" t="n">
         <f aca="false">P51+$B$18</f>
-        <v>75631.9775726025</v>
+        <v>70972.1198653134</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="34" t="n">
-        <v>46600</v>
+        <v>46539</v>
       </c>
       <c r="B52" s="21" t="n">
-        <f aca="false">IF(A52&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A52&gt;$B$38,$B$39,0)+IF(A52&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A52&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A52&gt;$B$40,$B$41,0)+IF(A52&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C52" s="12" t="n">
-        <f aca="false">IF(A52=$B$37,$B$26-$B$29,0)-IF(A52=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A52=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A52=$B$39,$B$26-$B$29,0)-IF(A52=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A52=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D52" s="12" t="n">
         <f aca="false">B52+C52</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E52" s="12" t="n">
         <f aca="false">H51</f>
@@ -6064,15 +5916,15 @@
       </c>
       <c r="N52" s="12" t="n">
         <f aca="false">P51</f>
-        <v>59371.2275726024</v>
+        <v>54711.3698653134</v>
       </c>
       <c r="O52" s="12" t="n">
         <f aca="false">MIN(D52-G52-L52,MAX($B$15-$B$18-N52,0))</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="P52" s="12" t="n">
         <f aca="false">N52+O52</f>
-        <v>61888.2629892691</v>
+        <v>57280.4631986467</v>
       </c>
       <c r="Q52" s="5" t="n">
         <f aca="false">IF(H52&lt;=0.005,1,0)</f>
@@ -6100,24 +5952,24 @@
       </c>
       <c r="W52" s="12" t="n">
         <f aca="false">P52+$B$18</f>
-        <v>78149.0129892691</v>
+        <v>73541.2131986467</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="34" t="n">
-        <v>46631</v>
+        <v>46569</v>
       </c>
       <c r="B53" s="21" t="n">
-        <f aca="false">IF(A53&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A53&gt;$B$38,$B$39,0)+IF(A53&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A53&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A53&gt;$B$40,$B$41,0)+IF(A53&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C53" s="12" t="n">
-        <f aca="false">IF(A53=$B$37,$B$26-$B$29,0)-IF(A53=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A53=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A53=$B$39,$B$26-$B$29,0)-IF(A53=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A53=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D53" s="12" t="n">
         <f aca="false">B53+C53</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E53" s="12" t="n">
         <f aca="false">H52</f>
@@ -6157,15 +6009,15 @@
       </c>
       <c r="N53" s="12" t="n">
         <f aca="false">P52</f>
-        <v>61888.2629892691</v>
+        <v>57280.4631986467</v>
       </c>
       <c r="O53" s="12" t="n">
         <f aca="false">MIN(D53-G53-L53,MAX($B$15-$B$18-N53,0))</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="P53" s="12" t="n">
         <f aca="false">N53+O53</f>
-        <v>64405.2984059358</v>
+        <v>59849.55653198</v>
       </c>
       <c r="Q53" s="5" t="n">
         <f aca="false">IF(H53&lt;=0.005,1,0)</f>
@@ -6193,24 +6045,24 @@
       </c>
       <c r="W53" s="12" t="n">
         <f aca="false">P53+$B$18</f>
-        <v>80666.0484059358</v>
+        <v>76110.30653198</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="34" t="n">
-        <v>46661</v>
+        <v>46600</v>
       </c>
       <c r="B54" s="21" t="n">
-        <f aca="false">IF(A54&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A54&gt;$B$38,$B$39,0)+IF(A54&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A54&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A54&gt;$B$40,$B$41,0)+IF(A54&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C54" s="12" t="n">
-        <f aca="false">IF(A54=$B$37,$B$26-$B$29,0)-IF(A54=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A54=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A54=$B$39,$B$26-$B$29,0)-IF(A54=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A54=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D54" s="12" t="n">
         <f aca="false">B54+C54</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E54" s="12" t="n">
         <f aca="false">H53</f>
@@ -6250,15 +6102,15 @@
       </c>
       <c r="N54" s="12" t="n">
         <f aca="false">P53</f>
-        <v>64405.2984059358</v>
+        <v>59849.55653198</v>
       </c>
       <c r="O54" s="12" t="n">
         <f aca="false">MIN(D54-G54-L54,MAX($B$15-$B$18-N54,0))</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="P54" s="12" t="n">
         <f aca="false">N54+O54</f>
-        <v>66922.3338226025</v>
+        <v>62418.6498653134</v>
       </c>
       <c r="Q54" s="5" t="n">
         <f aca="false">IF(H54&lt;=0.005,1,0)</f>
@@ -6286,24 +6138,24 @@
       </c>
       <c r="W54" s="12" t="n">
         <f aca="false">P54+$B$18</f>
-        <v>83183.0838226025</v>
+        <v>78679.3998653134</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="34" t="n">
-        <v>46692</v>
+        <v>46631</v>
       </c>
       <c r="B55" s="21" t="n">
-        <f aca="false">IF(A55&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A55&gt;$B$38,$B$39,0)+IF(A55&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A55&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A55&gt;$B$40,$B$41,0)+IF(A55&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C55" s="12" t="n">
-        <f aca="false">IF(A55=$B$37,$B$26-$B$29,0)-IF(A55=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A55=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A55=$B$39,$B$26-$B$29,0)-IF(A55=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A55=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D55" s="12" t="n">
         <f aca="false">B55+C55</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E55" s="12" t="n">
         <f aca="false">H54</f>
@@ -6343,15 +6195,15 @@
       </c>
       <c r="N55" s="12" t="n">
         <f aca="false">P54</f>
-        <v>66922.3338226025</v>
+        <v>62418.6498653134</v>
       </c>
       <c r="O55" s="12" t="n">
         <f aca="false">MIN(D55-G55-L55,MAX($B$15-$B$18-N55,0))</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="P55" s="12" t="n">
         <f aca="false">N55+O55</f>
-        <v>69439.3692392691</v>
+        <v>64987.7431986467</v>
       </c>
       <c r="Q55" s="5" t="n">
         <f aca="false">IF(H55&lt;=0.005,1,0)</f>
@@ -6379,24 +6231,24 @@
       </c>
       <c r="W55" s="12" t="n">
         <f aca="false">P55+$B$18</f>
-        <v>85700.1192392691</v>
+        <v>81248.4931986467</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="34" t="n">
-        <v>46722</v>
+        <v>46661</v>
       </c>
       <c r="B56" s="21" t="n">
-        <f aca="false">IF(A56&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A56&gt;$B$38,$B$39,0)+IF(A56&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A56&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A56&gt;$B$40,$B$41,0)+IF(A56&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C56" s="12" t="n">
-        <f aca="false">IF(A56=$B$37,$B$26-$B$29,0)-IF(A56=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A56=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A56=$B$39,$B$26-$B$29,0)-IF(A56=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A56=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D56" s="12" t="n">
         <f aca="false">B56+C56</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E56" s="12" t="n">
         <f aca="false">H55</f>
@@ -6436,15 +6288,15 @@
       </c>
       <c r="N56" s="12" t="n">
         <f aca="false">P55</f>
-        <v>69439.3692392691</v>
+        <v>64987.7431986467</v>
       </c>
       <c r="O56" s="12" t="n">
         <f aca="false">MIN(D56-G56-L56,MAX($B$15-$B$18-N56,0))</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="P56" s="12" t="n">
         <f aca="false">N56+O56</f>
-        <v>71956.4046559358</v>
+        <v>67556.83653198</v>
       </c>
       <c r="Q56" s="5" t="n">
         <f aca="false">IF(H56&lt;=0.005,1,0)</f>
@@ -6472,24 +6324,24 @@
       </c>
       <c r="W56" s="12" t="n">
         <f aca="false">P56+$B$18</f>
-        <v>88217.1546559358</v>
+        <v>83817.58653198</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="34" t="n">
-        <v>46753</v>
+        <v>46692</v>
       </c>
       <c r="B57" s="21" t="n">
-        <f aca="false">IF(A57&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A57&gt;$B$38,$B$39,0)+IF(A57&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A57&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A57&gt;$B$40,$B$41,0)+IF(A57&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C57" s="12" t="n">
-        <f aca="false">IF(A57=$B$37,$B$26-$B$29,0)-IF(A57=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A57=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A57=$B$39,$B$26-$B$29,0)-IF(A57=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A57=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D57" s="12" t="n">
         <f aca="false">B57+C57</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E57" s="12" t="n">
         <f aca="false">H56</f>
@@ -6529,15 +6381,15 @@
       </c>
       <c r="N57" s="12" t="n">
         <f aca="false">P56</f>
-        <v>71956.4046559358</v>
+        <v>67556.83653198</v>
       </c>
       <c r="O57" s="12" t="n">
         <f aca="false">MIN(D57-G57-L57,MAX($B$15-$B$18-N57,0))</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="P57" s="12" t="n">
         <f aca="false">N57+O57</f>
-        <v>74473.4400726025</v>
+        <v>70125.9298653134</v>
       </c>
       <c r="Q57" s="5" t="n">
         <f aca="false">IF(H57&lt;=0.005,1,0)</f>
@@ -6565,24 +6417,24 @@
       </c>
       <c r="W57" s="12" t="n">
         <f aca="false">P57+$B$18</f>
-        <v>90734.1900726025</v>
+        <v>86386.6798653134</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="34" t="n">
-        <v>46784</v>
+        <v>46722</v>
       </c>
       <c r="B58" s="21" t="n">
-        <f aca="false">IF(A58&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A58&gt;$B$38,$B$39,0)+IF(A58&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A58&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A58&gt;$B$40,$B$41,0)+IF(A58&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C58" s="12" t="n">
-        <f aca="false">IF(A58=$B$37,$B$26-$B$29,0)-IF(A58=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A58=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A58=$B$39,$B$26-$B$29,0)-IF(A58=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A58=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D58" s="12" t="n">
         <f aca="false">B58+C58</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E58" s="12" t="n">
         <f aca="false">H57</f>
@@ -6622,15 +6474,15 @@
       </c>
       <c r="N58" s="12" t="n">
         <f aca="false">P57</f>
-        <v>74473.4400726025</v>
+        <v>70125.9298653134</v>
       </c>
       <c r="O58" s="12" t="n">
         <f aca="false">MIN(D58-G58-L58,MAX($B$15-$B$18-N58,0))</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="P58" s="12" t="n">
         <f aca="false">N58+O58</f>
-        <v>76990.4754892691</v>
+        <v>72695.0231986467</v>
       </c>
       <c r="Q58" s="5" t="n">
         <f aca="false">IF(H58&lt;=0.005,1,0)</f>
@@ -6658,24 +6510,24 @@
       </c>
       <c r="W58" s="12" t="n">
         <f aca="false">P58+$B$18</f>
-        <v>93251.2254892691</v>
+        <v>88955.7731986467</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="34" t="n">
-        <v>46813</v>
+        <v>46753</v>
       </c>
       <c r="B59" s="21" t="n">
-        <f aca="false">IF(A59&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A59&gt;$B$38,$B$39,0)+IF(A59&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A59&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A59&gt;$B$40,$B$41,0)+IF(A59&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C59" s="12" t="n">
-        <f aca="false">IF(A59=$B$37,$B$26-$B$29,0)-IF(A59=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A59=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A59=$B$39,$B$26-$B$29,0)-IF(A59=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A59=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D59" s="12" t="n">
         <f aca="false">B59+C59</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E59" s="12" t="n">
         <f aca="false">H58</f>
@@ -6715,15 +6567,15 @@
       </c>
       <c r="N59" s="12" t="n">
         <f aca="false">P58</f>
-        <v>76990.4754892691</v>
+        <v>72695.0231986467</v>
       </c>
       <c r="O59" s="12" t="n">
         <f aca="false">MIN(D59-G59-L59,MAX($B$15-$B$18-N59,0))</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="P59" s="12" t="n">
         <f aca="false">N59+O59</f>
-        <v>79507.5109059358</v>
+        <v>75264.1165319801</v>
       </c>
       <c r="Q59" s="5" t="n">
         <f aca="false">IF(H59&lt;=0.005,1,0)</f>
@@ -6751,24 +6603,24 @@
       </c>
       <c r="W59" s="12" t="n">
         <f aca="false">P59+$B$18</f>
-        <v>95768.2609059358</v>
+        <v>91524.8665319801</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="34" t="n">
-        <v>46844</v>
+        <v>46784</v>
       </c>
       <c r="B60" s="21" t="n">
-        <f aca="false">IF(A60&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A60&gt;$B$38,$B$39,0)+IF(A60&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A60&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A60&gt;$B$40,$B$41,0)+IF(A60&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C60" s="12" t="n">
-        <f aca="false">IF(A60=$B$37,$B$26-$B$29,0)-IF(A60=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A60=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A60=$B$39,$B$26-$B$29,0)-IF(A60=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A60=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D60" s="12" t="n">
         <f aca="false">B60+C60</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E60" s="12" t="n">
         <f aca="false">H59</f>
@@ -6808,15 +6660,15 @@
       </c>
       <c r="N60" s="12" t="n">
         <f aca="false">P59</f>
-        <v>79507.5109059358</v>
+        <v>75264.1165319801</v>
       </c>
       <c r="O60" s="12" t="n">
         <f aca="false">MIN(D60-G60-L60,MAX($B$15-$B$18-N60,0))</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="P60" s="12" t="n">
         <f aca="false">N60+O60</f>
-        <v>82024.5463226024</v>
+        <v>77833.2098653134</v>
       </c>
       <c r="Q60" s="5" t="n">
         <f aca="false">IF(H60&lt;=0.005,1,0)</f>
@@ -6844,24 +6696,24 @@
       </c>
       <c r="W60" s="12" t="n">
         <f aca="false">P60+$B$18</f>
-        <v>98285.2963226024</v>
+        <v>94093.9598653134</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="34" t="n">
-        <v>46874</v>
+        <v>46813</v>
       </c>
       <c r="B61" s="21" t="n">
-        <f aca="false">IF(A61&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A61&gt;$B$38,$B$39,0)+IF(A61&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A61&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A61&gt;$B$40,$B$41,0)+IF(A61&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C61" s="12" t="n">
-        <f aca="false">IF(A61=$B$37,$B$26-$B$29,0)-IF(A61=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A61=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A61=$B$39,$B$26-$B$29,0)-IF(A61=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A61=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D61" s="12" t="n">
         <f aca="false">B61+C61</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E61" s="12" t="n">
         <f aca="false">H60</f>
@@ -6901,15 +6753,15 @@
       </c>
       <c r="N61" s="12" t="n">
         <f aca="false">P60</f>
-        <v>82024.5463226024</v>
+        <v>77833.2098653134</v>
       </c>
       <c r="O61" s="12" t="n">
         <f aca="false">MIN(D61-G61-L61,MAX($B$15-$B$18-N61,0))</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="P61" s="12" t="n">
         <f aca="false">N61+O61</f>
-        <v>84541.5817392691</v>
+        <v>80402.3031986467</v>
       </c>
       <c r="Q61" s="5" t="n">
         <f aca="false">IF(H61&lt;=0.005,1,0)</f>
@@ -6937,24 +6789,24 @@
       </c>
       <c r="W61" s="12" t="n">
         <f aca="false">P61+$B$18</f>
-        <v>100802.331739269</v>
+        <v>96663.0531986467</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="34" t="n">
-        <v>46905</v>
+        <v>46844</v>
       </c>
       <c r="B62" s="21" t="n">
-        <f aca="false">IF(A62&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A62&gt;$B$38,$B$39,0)+IF(A62&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A62&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A62&gt;$B$40,$B$41,0)+IF(A62&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C62" s="12" t="n">
-        <f aca="false">IF(A62=$B$37,$B$26-$B$29,0)-IF(A62=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A62=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A62=$B$39,$B$26-$B$29,0)-IF(A62=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A62=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D62" s="12" t="n">
         <f aca="false">B62+C62</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E62" s="12" t="n">
         <f aca="false">H61</f>
@@ -6994,15 +6846,15 @@
       </c>
       <c r="N62" s="12" t="n">
         <f aca="false">P61</f>
-        <v>84541.5817392691</v>
+        <v>80402.3031986467</v>
       </c>
       <c r="O62" s="12" t="n">
         <f aca="false">MIN(D62-G62-L62,MAX($B$15-$B$18-N62,0))</f>
-        <v>39.6682607308903</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="P62" s="12" t="n">
         <f aca="false">N62+O62</f>
-        <v>84581.25</v>
+        <v>82971.3965319801</v>
       </c>
       <c r="Q62" s="5" t="n">
         <f aca="false">IF(H62&lt;=0.005,1,0)</f>
@@ -7022,32 +6874,32 @@
       </c>
       <c r="U62" s="5" t="n">
         <f aca="false">IF(P62+$B$18&gt;=$B$15-0.5,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V62" s="12" t="n">
         <f aca="false">MAX(D62-G62-L62,0)-MAX(O62,0)</f>
-        <v>2477.36715593578</v>
+        <v>0</v>
       </c>
       <c r="W62" s="12" t="n">
         <f aca="false">P62+$B$18</f>
-        <v>100842</v>
+        <v>99232.1465319801</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="34" t="n">
-        <v>46935</v>
+        <v>46874</v>
       </c>
       <c r="B63" s="21" t="n">
-        <f aca="false">IF(A63&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A63&gt;$B$38,$B$39,0)+IF(A63&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A63&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A63&gt;$B$40,$B$41,0)+IF(A63&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C63" s="12" t="n">
-        <f aca="false">IF(A63=$B$37,$B$26-$B$29,0)-IF(A63=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A63=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A63=$B$39,$B$26-$B$29,0)-IF(A63=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A63=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D63" s="12" t="n">
         <f aca="false">B63+C63</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E63" s="12" t="n">
         <f aca="false">H62</f>
@@ -7087,11 +6939,11 @@
       </c>
       <c r="N63" s="12" t="n">
         <f aca="false">P62</f>
-        <v>84581.25</v>
+        <v>82971.3965319801</v>
       </c>
       <c r="O63" s="12" t="n">
         <f aca="false">MIN(D63-G63-L63,MAX($B$15-$B$18-N63,0))</f>
-        <v>0</v>
+        <v>1609.85346801994</v>
       </c>
       <c r="P63" s="12" t="n">
         <f aca="false">N63+O63</f>
@@ -7119,7 +6971,7 @@
       </c>
       <c r="V63" s="12" t="n">
         <f aca="false">MAX(D63-G63-L63,0)-MAX(O63,0)</f>
-        <v>2517.03541666667</v>
+        <v>959.239865313398</v>
       </c>
       <c r="W63" s="12" t="n">
         <f aca="false">P63+$B$18</f>
@@ -7128,19 +6980,19 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="34" t="n">
-        <v>46966</v>
+        <v>46905</v>
       </c>
       <c r="B64" s="21" t="n">
-        <f aca="false">IF(A64&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A64&gt;$B$38,$B$39,0)+IF(A64&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A64&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A64&gt;$B$40,$B$41,0)+IF(A64&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C64" s="12" t="n">
-        <f aca="false">IF(A64=$B$37,$B$26-$B$29,0)-IF(A64=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A64=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A64=$B$39,$B$26-$B$29,0)-IF(A64=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A64=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D64" s="12" t="n">
         <f aca="false">B64+C64</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E64" s="12" t="n">
         <f aca="false">H63</f>
@@ -7212,7 +7064,7 @@
       </c>
       <c r="V64" s="12" t="n">
         <f aca="false">MAX(D64-G64-L64,0)-MAX(O64,0)</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="W64" s="12" t="n">
         <f aca="false">P64+$B$18</f>
@@ -7221,19 +7073,19 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="34" t="n">
-        <v>46997</v>
+        <v>46935</v>
       </c>
       <c r="B65" s="21" t="n">
-        <f aca="false">IF(A65&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A65&gt;$B$38,$B$39,0)+IF(A65&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A65&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A65&gt;$B$40,$B$41,0)+IF(A65&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C65" s="12" t="n">
-        <f aca="false">IF(A65=$B$37,$B$26-$B$29,0)-IF(A65=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A65=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A65=$B$39,$B$26-$B$29,0)-IF(A65=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A65=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D65" s="12" t="n">
         <f aca="false">B65+C65</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E65" s="12" t="n">
         <f aca="false">H64</f>
@@ -7305,7 +7157,7 @@
       </c>
       <c r="V65" s="12" t="n">
         <f aca="false">MAX(D65-G65-L65,0)-MAX(O65,0)</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="W65" s="12" t="n">
         <f aca="false">P65+$B$18</f>
@@ -7314,19 +7166,19 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="34" t="n">
-        <v>47027</v>
+        <v>46966</v>
       </c>
       <c r="B66" s="21" t="n">
-        <f aca="false">IF(A66&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A66&gt;$B$38,$B$39,0)+IF(A66&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A66&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A66&gt;$B$40,$B$41,0)+IF(A66&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C66" s="12" t="n">
-        <f aca="false">IF(A66=$B$37,$B$26-$B$29,0)-IF(A66=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A66=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A66=$B$39,$B$26-$B$29,0)-IF(A66=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A66=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D66" s="12" t="n">
         <f aca="false">B66+C66</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E66" s="12" t="n">
         <f aca="false">H65</f>
@@ -7398,7 +7250,7 @@
       </c>
       <c r="V66" s="12" t="n">
         <f aca="false">MAX(D66-G66-L66,0)-MAX(O66,0)</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="W66" s="12" t="n">
         <f aca="false">P66+$B$18</f>
@@ -7407,19 +7259,19 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="34" t="n">
-        <v>47058</v>
+        <v>46997</v>
       </c>
       <c r="B67" s="21" t="n">
-        <f aca="false">IF(A67&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A67&gt;$B$38,$B$39,0)+IF(A67&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A67&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A67&gt;$B$40,$B$41,0)+IF(A67&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C67" s="12" t="n">
-        <f aca="false">IF(A67=$B$37,$B$26-$B$29,0)-IF(A67=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A67=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A67=$B$39,$B$26-$B$29,0)-IF(A67=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A67=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D67" s="12" t="n">
         <f aca="false">B67+C67</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E67" s="12" t="n">
         <f aca="false">H66</f>
@@ -7491,7 +7343,7 @@
       </c>
       <c r="V67" s="12" t="n">
         <f aca="false">MAX(D67-G67-L67,0)-MAX(O67,0)</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="W67" s="12" t="n">
         <f aca="false">P67+$B$18</f>
@@ -7500,19 +7352,19 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="34" t="n">
-        <v>47088</v>
+        <v>47027</v>
       </c>
       <c r="B68" s="21" t="n">
-        <f aca="false">IF(A68&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A68&gt;$B$38,$B$39,0)+IF(A68&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A68&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A68&gt;$B$40,$B$41,0)+IF(A68&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C68" s="12" t="n">
-        <f aca="false">IF(A68=$B$37,$B$26-$B$29,0)-IF(A68=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A68=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A68=$B$39,$B$26-$B$29,0)-IF(A68=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A68=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D68" s="12" t="n">
         <f aca="false">B68+C68</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E68" s="12" t="n">
         <f aca="false">H67</f>
@@ -7584,7 +7436,7 @@
       </c>
       <c r="V68" s="12" t="n">
         <f aca="false">MAX(D68-G68-L68,0)-MAX(O68,0)</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="W68" s="12" t="n">
         <f aca="false">P68+$B$18</f>
@@ -7593,19 +7445,19 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="34" t="n">
-        <v>47119</v>
+        <v>47058</v>
       </c>
       <c r="B69" s="21" t="n">
-        <f aca="false">IF(A69&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A69&gt;$B$38,$B$39,0)+IF(A69&gt;=$B$33,$B$35,0)</f>
-        <v>2517.03541666667</v>
+        <f aca="false">IF(A69&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A69&gt;$B$40,$B$41,0)+IF(A69&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C69" s="12" t="n">
-        <f aca="false">IF(A69=$B$37,$B$26-$B$29,0)-IF(A69=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A69=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A69=$B$39,$B$26-$B$29,0)-IF(A69=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A69=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D69" s="12" t="n">
         <f aca="false">B69+C69</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E69" s="12" t="n">
         <f aca="false">H68</f>
@@ -7677,7 +7529,7 @@
       </c>
       <c r="V69" s="12" t="n">
         <f aca="false">MAX(D69-G69-L69,0)-MAX(O69,0)</f>
-        <v>2517.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="W69" s="12" t="n">
         <f aca="false">P69+$B$18</f>
@@ -7686,19 +7538,19 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="34" t="n">
-        <v>47150</v>
+        <v>47088</v>
       </c>
       <c r="B70" s="21" t="n">
-        <f aca="false">IF(A70&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A70&gt;$B$38,$B$39,0)+IF(A70&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A70&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A70&gt;$B$40,$B$41,0)+IF(A70&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C70" s="12" t="n">
-        <f aca="false">IF(A70=$B$37,$B$26-$B$29,0)-IF(A70=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A70=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A70=$B$39,$B$26-$B$29,0)-IF(A70=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A70=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D70" s="12" t="n">
         <f aca="false">B70+C70</f>
-        <v>2859.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E70" s="12" t="n">
         <f aca="false">H69</f>
@@ -7770,7 +7622,7 @@
       </c>
       <c r="V70" s="12" t="n">
         <f aca="false">MAX(D70-G70-L70,0)-MAX(O70,0)</f>
-        <v>2859.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="W70" s="12" t="n">
         <f aca="false">P70+$B$18</f>
@@ -7779,19 +7631,19 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="34" t="n">
-        <v>47178</v>
+        <v>47119</v>
       </c>
       <c r="B71" s="21" t="n">
-        <f aca="false">IF(A71&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A71&gt;$B$38,$B$39,0)+IF(A71&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A71&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A71&gt;$B$40,$B$41,0)+IF(A71&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C71" s="12" t="n">
-        <f aca="false">IF(A71=$B$37,$B$26-$B$29,0)-IF(A71=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A71=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A71=$B$39,$B$26-$B$29,0)-IF(A71=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A71=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D71" s="12" t="n">
         <f aca="false">B71+C71</f>
-        <v>2859.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E71" s="12" t="n">
         <f aca="false">H70</f>
@@ -7863,7 +7715,7 @@
       </c>
       <c r="V71" s="12" t="n">
         <f aca="false">MAX(D71-G71-L71,0)-MAX(O71,0)</f>
-        <v>2859.03541666667</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="W71" s="12" t="n">
         <f aca="false">P71+$B$18</f>
@@ -7872,19 +7724,19 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="34" t="n">
-        <v>47209</v>
+        <v>47150</v>
       </c>
       <c r="B72" s="21" t="n">
-        <f aca="false">IF(A72&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A72&gt;$B$38,$B$39,0)+IF(A72&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A72&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A72&gt;$B$40,$B$41,0)+IF(A72&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C72" s="12" t="n">
-        <f aca="false">IF(A72=$B$37,$B$26-$B$29,0)-IF(A72=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A72=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A72=$B$39,$B$26-$B$29,0)-IF(A72=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A72=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D72" s="12" t="n">
         <f aca="false">B72+C72</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E72" s="12" t="n">
         <f aca="false">H71</f>
@@ -7956,7 +7808,7 @@
       </c>
       <c r="V72" s="12" t="n">
         <f aca="false">MAX(D72-G72-L72,0)-MAX(O72,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W72" s="12" t="n">
         <f aca="false">P72+$B$18</f>
@@ -7965,19 +7817,19 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="34" t="n">
-        <v>47239</v>
+        <v>47178</v>
       </c>
       <c r="B73" s="21" t="n">
-        <f aca="false">IF(A73&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A73&gt;$B$38,$B$39,0)+IF(A73&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A73&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A73&gt;$B$40,$B$41,0)+IF(A73&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C73" s="12" t="n">
-        <f aca="false">IF(A73=$B$37,$B$26-$B$29,0)-IF(A73=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A73=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A73=$B$39,$B$26-$B$29,0)-IF(A73=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A73=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D73" s="12" t="n">
         <f aca="false">B73+C73</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E73" s="12" t="n">
         <f aca="false">H72</f>
@@ -8049,7 +7901,7 @@
       </c>
       <c r="V73" s="12" t="n">
         <f aca="false">MAX(D73-G73-L73,0)-MAX(O73,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W73" s="12" t="n">
         <f aca="false">P73+$B$18</f>
@@ -8058,19 +7910,19 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="34" t="n">
-        <v>47270</v>
+        <v>47209</v>
       </c>
       <c r="B74" s="21" t="n">
-        <f aca="false">IF(A74&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A74&gt;$B$38,$B$39,0)+IF(A74&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A74&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A74&gt;$B$40,$B$41,0)+IF(A74&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C74" s="12" t="n">
-        <f aca="false">IF(A74=$B$37,$B$26-$B$29,0)-IF(A74=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A74=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A74=$B$39,$B$26-$B$29,0)-IF(A74=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A74=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D74" s="12" t="n">
         <f aca="false">B74+C74</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E74" s="12" t="n">
         <f aca="false">H73</f>
@@ -8142,7 +7994,7 @@
       </c>
       <c r="V74" s="12" t="n">
         <f aca="false">MAX(D74-G74-L74,0)-MAX(O74,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W74" s="12" t="n">
         <f aca="false">P74+$B$18</f>
@@ -8151,19 +8003,19 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="34" t="n">
-        <v>47300</v>
+        <v>47239</v>
       </c>
       <c r="B75" s="21" t="n">
-        <f aca="false">IF(A75&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A75&gt;$B$38,$B$39,0)+IF(A75&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A75&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A75&gt;$B$40,$B$41,0)+IF(A75&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C75" s="12" t="n">
-        <f aca="false">IF(A75=$B$37,$B$26-$B$29,0)-IF(A75=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A75=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A75=$B$39,$B$26-$B$29,0)-IF(A75=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A75=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D75" s="12" t="n">
         <f aca="false">B75+C75</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E75" s="12" t="n">
         <f aca="false">H74</f>
@@ -8235,7 +8087,7 @@
       </c>
       <c r="V75" s="12" t="n">
         <f aca="false">MAX(D75-G75-L75,0)-MAX(O75,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W75" s="12" t="n">
         <f aca="false">P75+$B$18</f>
@@ -8244,19 +8096,19 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="34" t="n">
-        <v>47331</v>
+        <v>47270</v>
       </c>
       <c r="B76" s="21" t="n">
-        <f aca="false">IF(A76&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A76&gt;$B$38,$B$39,0)+IF(A76&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A76&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A76&gt;$B$40,$B$41,0)+IF(A76&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C76" s="12" t="n">
-        <f aca="false">IF(A76=$B$37,$B$26-$B$29,0)-IF(A76=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A76=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A76=$B$39,$B$26-$B$29,0)-IF(A76=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A76=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D76" s="12" t="n">
         <f aca="false">B76+C76</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E76" s="12" t="n">
         <f aca="false">H75</f>
@@ -8328,7 +8180,7 @@
       </c>
       <c r="V76" s="12" t="n">
         <f aca="false">MAX(D76-G76-L76,0)-MAX(O76,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W76" s="12" t="n">
         <f aca="false">P76+$B$18</f>
@@ -8337,19 +8189,19 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="34" t="n">
-        <v>47362</v>
+        <v>47300</v>
       </c>
       <c r="B77" s="21" t="n">
-        <f aca="false">IF(A77&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A77&gt;$B$38,$B$39,0)+IF(A77&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A77&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A77&gt;$B$40,$B$41,0)+IF(A77&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C77" s="12" t="n">
-        <f aca="false">IF(A77=$B$37,$B$26-$B$29,0)-IF(A77=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A77=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A77=$B$39,$B$26-$B$29,0)-IF(A77=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A77=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D77" s="12" t="n">
         <f aca="false">B77+C77</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E77" s="12" t="n">
         <f aca="false">H76</f>
@@ -8421,7 +8273,7 @@
       </c>
       <c r="V77" s="12" t="n">
         <f aca="false">MAX(D77-G77-L77,0)-MAX(O77,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W77" s="12" t="n">
         <f aca="false">P77+$B$18</f>
@@ -8430,19 +8282,19 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="34" t="n">
-        <v>47392</v>
+        <v>47331</v>
       </c>
       <c r="B78" s="21" t="n">
-        <f aca="false">IF(A78&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A78&gt;$B$38,$B$39,0)+IF(A78&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A78&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A78&gt;$B$40,$B$41,0)+IF(A78&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C78" s="12" t="n">
-        <f aca="false">IF(A78=$B$37,$B$26-$B$29,0)-IF(A78=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A78=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A78=$B$39,$B$26-$B$29,0)-IF(A78=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A78=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D78" s="12" t="n">
         <f aca="false">B78+C78</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E78" s="12" t="n">
         <f aca="false">H77</f>
@@ -8514,7 +8366,7 @@
       </c>
       <c r="V78" s="12" t="n">
         <f aca="false">MAX(D78-G78-L78,0)-MAX(O78,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W78" s="12" t="n">
         <f aca="false">P78+$B$18</f>
@@ -8523,19 +8375,19 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="34" t="n">
-        <v>47423</v>
+        <v>47362</v>
       </c>
       <c r="B79" s="21" t="n">
-        <f aca="false">IF(A79&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A79&gt;$B$38,$B$39,0)+IF(A79&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A79&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A79&gt;$B$40,$B$41,0)+IF(A79&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C79" s="12" t="n">
-        <f aca="false">IF(A79=$B$37,$B$26-$B$29,0)-IF(A79=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A79=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A79=$B$39,$B$26-$B$29,0)-IF(A79=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A79=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D79" s="12" t="n">
         <f aca="false">B79+C79</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E79" s="12" t="n">
         <f aca="false">H78</f>
@@ -8607,7 +8459,7 @@
       </c>
       <c r="V79" s="12" t="n">
         <f aca="false">MAX(D79-G79-L79,0)-MAX(O79,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W79" s="12" t="n">
         <f aca="false">P79+$B$18</f>
@@ -8616,19 +8468,19 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="34" t="n">
-        <v>47453</v>
+        <v>47392</v>
       </c>
       <c r="B80" s="21" t="n">
-        <f aca="false">IF(A80&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A80&gt;$B$38,$B$39,0)+IF(A80&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A80&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A80&gt;$B$40,$B$41,0)+IF(A80&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C80" s="12" t="n">
-        <f aca="false">IF(A80=$B$37,$B$26-$B$29,0)-IF(A80=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A80=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A80=$B$39,$B$26-$B$29,0)-IF(A80=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A80=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D80" s="12" t="n">
         <f aca="false">B80+C80</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E80" s="12" t="n">
         <f aca="false">H79</f>
@@ -8700,7 +8552,7 @@
       </c>
       <c r="V80" s="12" t="n">
         <f aca="false">MAX(D80-G80-L80,0)-MAX(O80,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W80" s="12" t="n">
         <f aca="false">P80+$B$18</f>
@@ -8709,19 +8561,19 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="34" t="n">
-        <v>47484</v>
+        <v>47423</v>
       </c>
       <c r="B81" s="21" t="n">
-        <f aca="false">IF(A81&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A81&gt;$B$38,$B$39,0)+IF(A81&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A81&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A81&gt;$B$40,$B$41,0)+IF(A81&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C81" s="12" t="n">
-        <f aca="false">IF(A81=$B$37,$B$26-$B$29,0)-IF(A81=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A81=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A81=$B$39,$B$26-$B$29,0)-IF(A81=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A81=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D81" s="12" t="n">
         <f aca="false">B81+C81</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E81" s="12" t="n">
         <f aca="false">H80</f>
@@ -8793,7 +8645,7 @@
       </c>
       <c r="V81" s="12" t="n">
         <f aca="false">MAX(D81-G81-L81,0)-MAX(O81,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W81" s="12" t="n">
         <f aca="false">P81+$B$18</f>
@@ -8802,19 +8654,19 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="34" t="n">
-        <v>47515</v>
+        <v>47453</v>
       </c>
       <c r="B82" s="21" t="n">
-        <f aca="false">IF(A82&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A82&gt;$B$38,$B$39,0)+IF(A82&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A82&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A82&gt;$B$40,$B$41,0)+IF(A82&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C82" s="12" t="n">
-        <f aca="false">IF(A82=$B$37,$B$26-$B$29,0)-IF(A82=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A82=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A82=$B$39,$B$26-$B$29,0)-IF(A82=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A82=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D82" s="12" t="n">
         <f aca="false">B82+C82</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E82" s="12" t="n">
         <f aca="false">H81</f>
@@ -8886,7 +8738,7 @@
       </c>
       <c r="V82" s="12" t="n">
         <f aca="false">MAX(D82-G82-L82,0)-MAX(O82,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W82" s="12" t="n">
         <f aca="false">P82+$B$18</f>
@@ -8895,19 +8747,19 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="34" t="n">
-        <v>47543</v>
+        <v>47484</v>
       </c>
       <c r="B83" s="21" t="n">
-        <f aca="false">IF(A83&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A83&gt;$B$38,$B$39,0)+IF(A83&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A83&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A83&gt;$B$40,$B$41,0)+IF(A83&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C83" s="12" t="n">
-        <f aca="false">IF(A83=$B$37,$B$26-$B$29,0)-IF(A83=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A83=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A83=$B$39,$B$26-$B$29,0)-IF(A83=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A83=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D83" s="12" t="n">
         <f aca="false">B83+C83</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E83" s="12" t="n">
         <f aca="false">H82</f>
@@ -8979,7 +8831,7 @@
       </c>
       <c r="V83" s="12" t="n">
         <f aca="false">MAX(D83-G83-L83,0)-MAX(O83,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W83" s="12" t="n">
         <f aca="false">P83+$B$18</f>
@@ -8988,19 +8840,19 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="34" t="n">
-        <v>47574</v>
+        <v>47515</v>
       </c>
       <c r="B84" s="21" t="n">
-        <f aca="false">IF(A84&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A84&gt;$B$38,$B$39,0)+IF(A84&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A84&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A84&gt;$B$40,$B$41,0)+IF(A84&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C84" s="12" t="n">
-        <f aca="false">IF(A84=$B$37,$B$26-$B$29,0)-IF(A84=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A84=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A84=$B$39,$B$26-$B$29,0)-IF(A84=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A84=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D84" s="12" t="n">
         <f aca="false">B84+C84</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E84" s="12" t="n">
         <f aca="false">H83</f>
@@ -9072,7 +8924,7 @@
       </c>
       <c r="V84" s="12" t="n">
         <f aca="false">MAX(D84-G84-L84,0)-MAX(O84,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W84" s="12" t="n">
         <f aca="false">P84+$B$18</f>
@@ -9081,19 +8933,19 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="34" t="n">
-        <v>47604</v>
+        <v>47543</v>
       </c>
       <c r="B85" s="21" t="n">
-        <f aca="false">IF(A85&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A85&gt;$B$38,$B$39,0)+IF(A85&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A85&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A85&gt;$B$40,$B$41,0)+IF(A85&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C85" s="12" t="n">
-        <f aca="false">IF(A85=$B$37,$B$26-$B$29,0)-IF(A85=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A85=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A85=$B$39,$B$26-$B$29,0)-IF(A85=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A85=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D85" s="12" t="n">
         <f aca="false">B85+C85</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E85" s="12" t="n">
         <f aca="false">H84</f>
@@ -9165,7 +9017,7 @@
       </c>
       <c r="V85" s="12" t="n">
         <f aca="false">MAX(D85-G85-L85,0)-MAX(O85,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W85" s="12" t="n">
         <f aca="false">P85+$B$18</f>
@@ -9174,19 +9026,19 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="34" t="n">
-        <v>47635</v>
+        <v>47574</v>
       </c>
       <c r="B86" s="21" t="n">
-        <f aca="false">IF(A86&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A86&gt;$B$38,$B$39,0)+IF(A86&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A86&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A86&gt;$B$40,$B$41,0)+IF(A86&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C86" s="12" t="n">
-        <f aca="false">IF(A86=$B$37,$B$26-$B$29,0)-IF(A86=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A86=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A86=$B$39,$B$26-$B$29,0)-IF(A86=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A86=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D86" s="12" t="n">
         <f aca="false">B86+C86</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E86" s="12" t="n">
         <f aca="false">H85</f>
@@ -9258,7 +9110,7 @@
       </c>
       <c r="V86" s="12" t="n">
         <f aca="false">MAX(D86-G86-L86,0)-MAX(O86,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W86" s="12" t="n">
         <f aca="false">P86+$B$18</f>
@@ -9267,19 +9119,19 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="34" t="n">
-        <v>47665</v>
+        <v>47604</v>
       </c>
       <c r="B87" s="21" t="n">
-        <f aca="false">IF(A87&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A87&gt;$B$38,$B$39,0)+IF(A87&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A87&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A87&gt;$B$40,$B$41,0)+IF(A87&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C87" s="12" t="n">
-        <f aca="false">IF(A87=$B$37,$B$26-$B$29,0)-IF(A87=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A87=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A87=$B$39,$B$26-$B$29,0)-IF(A87=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A87=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D87" s="12" t="n">
         <f aca="false">B87+C87</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E87" s="12" t="n">
         <f aca="false">H86</f>
@@ -9351,7 +9203,7 @@
       </c>
       <c r="V87" s="12" t="n">
         <f aca="false">MAX(D87-G87-L87,0)-MAX(O87,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W87" s="12" t="n">
         <f aca="false">P87+$B$18</f>
@@ -9360,19 +9212,19 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="34" t="n">
-        <v>47696</v>
+        <v>47635</v>
       </c>
       <c r="B88" s="21" t="n">
-        <f aca="false">IF(A88&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A88&gt;$B$38,$B$39,0)+IF(A88&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A88&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A88&gt;$B$40,$B$41,0)+IF(A88&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C88" s="12" t="n">
-        <f aca="false">IF(A88=$B$37,$B$26-$B$29,0)-IF(A88=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A88=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A88=$B$39,$B$26-$B$29,0)-IF(A88=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A88=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D88" s="12" t="n">
         <f aca="false">B88+C88</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E88" s="12" t="n">
         <f aca="false">H87</f>
@@ -9444,7 +9296,7 @@
       </c>
       <c r="V88" s="12" t="n">
         <f aca="false">MAX(D88-G88-L88,0)-MAX(O88,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W88" s="12" t="n">
         <f aca="false">P88+$B$18</f>
@@ -9453,19 +9305,19 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="34" t="n">
-        <v>47727</v>
+        <v>47665</v>
       </c>
       <c r="B89" s="21" t="n">
-        <f aca="false">IF(A89&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A89&gt;$B$38,$B$39,0)+IF(A89&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A89&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A89&gt;$B$40,$B$41,0)+IF(A89&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C89" s="12" t="n">
-        <f aca="false">IF(A89=$B$37,$B$26-$B$29,0)-IF(A89=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A89=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A89=$B$39,$B$26-$B$29,0)-IF(A89=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A89=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D89" s="12" t="n">
         <f aca="false">B89+C89</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E89" s="12" t="n">
         <f aca="false">H88</f>
@@ -9537,7 +9389,7 @@
       </c>
       <c r="V89" s="12" t="n">
         <f aca="false">MAX(D89-G89-L89,0)-MAX(O89,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W89" s="12" t="n">
         <f aca="false">P89+$B$18</f>
@@ -9546,19 +9398,19 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="34" t="n">
-        <v>47757</v>
+        <v>47696</v>
       </c>
       <c r="B90" s="21" t="n">
-        <f aca="false">IF(A90&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A90&gt;$B$38,$B$39,0)+IF(A90&gt;=$B$33,$B$35,0)</f>
-        <v>2859.03541666667</v>
+        <f aca="false">IF(A90&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A90&gt;$B$40,$B$41,0)+IF(A90&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
       </c>
       <c r="C90" s="12" t="n">
-        <f aca="false">IF(A90=$B$37,$B$26-$B$29,0)-IF(A90=DATE(YEAR($B$37),MONTH($B$37)+1,1),$B$28,0)+IF(A90=$B$33,$B$35*$B$34,0)+0</f>
+        <f aca="false">IF(A90=$B$39,$B$26-$B$29,0)-IF(A90=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A90=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D90" s="12" t="n">
         <f aca="false">B90+C90</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="E90" s="12" t="n">
         <f aca="false">H89</f>
@@ -9630,10 +9482,196 @@
       </c>
       <c r="V90" s="12" t="n">
         <f aca="false">MAX(D90-G90-L90,0)-MAX(O90,0)</f>
-        <v>2859.03541666667</v>
+        <v>2911.09333333334</v>
       </c>
       <c r="W90" s="12" t="n">
         <f aca="false">P90+$B$18</f>
+        <v>100842</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="34" t="n">
+        <v>47727</v>
+      </c>
+      <c r="B91" s="21" t="n">
+        <f aca="false">IF(A91&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A91&gt;$B$40,$B$41,0)+IF(A91&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
+      </c>
+      <c r="C91" s="12" t="n">
+        <f aca="false">IF(A91=$B$39,$B$26-$B$29,0)-IF(A91=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A91=$B$35,$B$37*$B$36,0)+0</f>
+        <v>0</v>
+      </c>
+      <c r="D91" s="12" t="n">
+        <f aca="false">B91+C91</f>
+        <v>2911.09333333334</v>
+      </c>
+      <c r="E91" s="12" t="n">
+        <f aca="false">H90</f>
+        <v>0</v>
+      </c>
+      <c r="F91" s="12" t="n">
+        <f aca="false">E91*$B$6/12</f>
+        <v>0</v>
+      </c>
+      <c r="G91" s="12" t="n">
+        <f aca="false">MIN(E91+F91,MAX(D91-K91,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H91" s="12" t="n">
+        <f aca="false">E91+F91-G91</f>
+        <v>0</v>
+      </c>
+      <c r="I91" s="12" t="n">
+        <f aca="false">M90</f>
+        <v>0</v>
+      </c>
+      <c r="J91" s="12" t="n">
+        <f aca="false">I91*$B$8/12</f>
+        <v>0</v>
+      </c>
+      <c r="K91" s="12" t="n">
+        <f aca="false">MIN(I91+J91,J91+$B$9*I91)</f>
+        <v>0</v>
+      </c>
+      <c r="L91" s="12" t="n">
+        <f aca="false">MIN(I91+J91,MAX(D91-G91,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M91" s="12" t="n">
+        <f aca="false">I91+J91-L91</f>
+        <v>0</v>
+      </c>
+      <c r="N91" s="12" t="n">
+        <f aca="false">P90</f>
+        <v>84581.25</v>
+      </c>
+      <c r="O91" s="12" t="n">
+        <f aca="false">MIN(D91-G91-L91,MAX($B$15-$B$18-N91,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P91" s="12" t="n">
+        <f aca="false">N91+O91</f>
+        <v>84581.25</v>
+      </c>
+      <c r="Q91" s="5" t="n">
+        <f aca="false">IF(H91&lt;=0.005,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="R91" s="5" t="n">
+        <f aca="false">IF(M91&lt;=0.005,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="S91" s="5" t="n">
+        <f aca="false">IF(AND(Q91=1,R91=1),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="T91" s="5" t="n">
+        <f aca="false">IF(P91&gt;=$B$20,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="U91" s="5" t="n">
+        <f aca="false">IF(P91+$B$18&gt;=$B$15-0.5,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="V91" s="12" t="n">
+        <f aca="false">MAX(D91-G91-L91,0)-MAX(O91,0)</f>
+        <v>2911.09333333334</v>
+      </c>
+      <c r="W91" s="12" t="n">
+        <f aca="false">P91+$B$18</f>
+        <v>100842</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="34" t="n">
+        <v>47757</v>
+      </c>
+      <c r="B92" s="21" t="n">
+        <f aca="false">IF(A92&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A92&gt;$B$40,$B$41,0)+IF(A92&gt;=$B$35,$B$37,0)+$B$32</f>
+        <v>2911.09333333334</v>
+      </c>
+      <c r="C92" s="12" t="n">
+        <f aca="false">IF(A92=$B$39,$B$26-$B$29,0)-IF(A92=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A92=$B$35,$B$37*$B$36,0)+0</f>
+        <v>0</v>
+      </c>
+      <c r="D92" s="12" t="n">
+        <f aca="false">B92+C92</f>
+        <v>2911.09333333334</v>
+      </c>
+      <c r="E92" s="12" t="n">
+        <f aca="false">H91</f>
+        <v>0</v>
+      </c>
+      <c r="F92" s="12" t="n">
+        <f aca="false">E92*$B$6/12</f>
+        <v>0</v>
+      </c>
+      <c r="G92" s="12" t="n">
+        <f aca="false">MIN(E92+F92,MAX(D92-K92,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H92" s="12" t="n">
+        <f aca="false">E92+F92-G92</f>
+        <v>0</v>
+      </c>
+      <c r="I92" s="12" t="n">
+        <f aca="false">M91</f>
+        <v>0</v>
+      </c>
+      <c r="J92" s="12" t="n">
+        <f aca="false">I92*$B$8/12</f>
+        <v>0</v>
+      </c>
+      <c r="K92" s="12" t="n">
+        <f aca="false">MIN(I92+J92,J92+$B$9*I92)</f>
+        <v>0</v>
+      </c>
+      <c r="L92" s="12" t="n">
+        <f aca="false">MIN(I92+J92,MAX(D92-G92,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M92" s="12" t="n">
+        <f aca="false">I92+J92-L92</f>
+        <v>0</v>
+      </c>
+      <c r="N92" s="12" t="n">
+        <f aca="false">P91</f>
+        <v>84581.25</v>
+      </c>
+      <c r="O92" s="12" t="n">
+        <f aca="false">MIN(D92-G92-L92,MAX($B$15-$B$18-N92,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P92" s="12" t="n">
+        <f aca="false">N92+O92</f>
+        <v>84581.25</v>
+      </c>
+      <c r="Q92" s="5" t="n">
+        <f aca="false">IF(H92&lt;=0.005,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="R92" s="5" t="n">
+        <f aca="false">IF(M92&lt;=0.005,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="S92" s="5" t="n">
+        <f aca="false">IF(AND(Q92=1,R92=1),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="T92" s="5" t="n">
+        <f aca="false">IF(P92&gt;=$B$20,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="U92" s="5" t="n">
+        <f aca="false">IF(P92+$B$18&gt;=$B$15-0.5,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="V92" s="12" t="n">
+        <f aca="false">MAX(D92-G92-L92,0)-MAX(O92,0)</f>
+        <v>2911.09333333334</v>
+      </c>
+      <c r="W92" s="12" t="n">
+        <f aca="false">P92+$B$18</f>
         <v>100842</v>
       </c>
     </row>
@@ -9664,12 +9702,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9677,48 +9715,48 @@
         <v>13</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="M4" s="10" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="N4" s="10" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -9736,7 +9774,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="B6" s="13" t="n">
         <v>17767.46</v>
@@ -9783,7 +9821,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="B7" s="13" t="n">
         <v>6410.38</v>
@@ -9830,7 +9868,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="B8" s="13" t="n">
         <v>1459.54</v>
@@ -9877,7 +9915,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="B9" s="17" t="n">
         <f aca="false">SUM(B6:B8)</f>
@@ -9934,7 +9972,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -9952,7 +9990,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="B12" s="13" t="n">
         <v>4300</v>
@@ -9999,7 +10037,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="B13" s="13" t="n">
         <v>32.71</v>
@@ -10046,7 +10084,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="B14" s="13" t="n">
         <v>0</v>
@@ -10093,7 +10131,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B15" s="13" t="n">
         <v>183.82</v>
@@ -10140,7 +10178,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="B16" s="13" t="n">
         <v>500</v>
@@ -10187,7 +10225,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="B17" s="17" t="n">
         <f aca="false">SUM(B12:B16)</f>
@@ -10244,7 +10282,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -10262,7 +10300,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="B20" s="13" t="n">
         <v>6857.93</v>
@@ -10356,7 +10394,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="B22" s="13" t="n">
         <v>1057.39</v>
@@ -10403,7 +10441,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="B23" s="13" t="n">
         <v>341.99</v>
@@ -10450,7 +10488,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="B24" s="13" t="n">
         <v>0</v>
@@ -10497,7 +10535,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="B25" s="13" t="n">
         <v>856.83</v>
@@ -10544,7 +10582,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="B26" s="13" t="n">
         <v>286.67</v>
@@ -10591,7 +10629,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="B27" s="13" t="n">
         <v>614</v>
@@ -10638,7 +10676,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="B28" s="13" t="n">
         <v>323.39</v>
@@ -10685,7 +10723,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="B29" s="13" t="n">
         <v>368.15</v>
@@ -10732,7 +10770,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="B30" s="13" t="n">
         <v>400.62</v>
@@ -10779,7 +10817,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="B31" s="13" t="n">
         <v>134.97</v>
@@ -10826,7 +10864,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="B32" s="13" t="n">
         <v>178.9</v>
@@ -10873,7 +10911,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="B33" s="13" t="n">
         <v>115.5</v>
@@ -10920,7 +10958,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="B34" s="13" t="n">
         <v>760</v>
@@ -10967,7 +11005,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="B35" s="13" t="n">
         <v>155</v>
@@ -11061,7 +11099,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="B37" s="13" t="n">
         <v>473.56</v>
@@ -11108,7 +11146,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="B38" s="13" t="n">
         <v>431.52</v>
@@ -11155,7 +11193,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="B39" s="13" t="n">
         <v>359.9</v>
@@ -11202,7 +11240,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="B40" s="13" t="n">
         <v>27.6</v>
@@ -11249,7 +11287,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="B41" s="13" t="n">
         <v>557.68</v>
@@ -11296,7 +11334,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="B42" s="13" t="n">
         <v>385.13</v>
@@ -11343,7 +11381,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="B43" s="13" t="n">
         <v>209</v>
@@ -11390,7 +11428,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="B44" s="13" t="n">
         <v>266.15</v>
@@ -11484,7 +11522,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="B46" s="13" t="n">
         <v>469.36</v>
@@ -11578,7 +11616,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="B48" s="13" t="n">
         <v>72.9</v>
@@ -11625,7 +11663,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="B49" s="13" t="n">
         <v>0.5</v>
@@ -11672,7 +11710,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="B50" s="13" t="n">
         <v>355.78</v>
@@ -11719,7 +11757,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="B51" s="13" t="n">
         <v>97.3</v>
@@ -11766,7 +11804,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B52" s="13" t="n">
         <v>129.41</v>
@@ -11813,7 +11851,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="B53" s="13" t="n">
         <v>465.78</v>
@@ -11860,7 +11898,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="B54" s="13" t="n">
         <v>240</v>
@@ -11907,7 +11945,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="B55" s="13" t="n">
         <v>729.5</v>
@@ -11954,7 +11992,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="B56" s="13" t="n">
         <v>2.25</v>
@@ -12001,7 +12039,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="B57" s="13" t="n">
         <v>0</v>
@@ -12048,7 +12086,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="B58" s="13" t="n">
         <v>127.73</v>
@@ -12095,7 +12133,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="15" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="B59" s="17" t="n">
         <f aca="false">SUM(B20:B58)</f>
@@ -12152,7 +12190,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="8" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="B61" s="28" t="n">
         <f aca="false">B17+B59</f>
@@ -12209,7 +12247,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="8" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="B62" s="28" t="n">
         <f aca="false">B9</f>
@@ -12266,7 +12304,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="8" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="B63" s="9" t="n">
         <f aca="false">B62-B61</f>
@@ -12352,35 +12390,35 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="H4" s="10" t="s">
         <v>20</v>
@@ -12388,10 +12426,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>72.97</v>
@@ -12401,25 +12439,25 @@
         <v>875.64</v>
       </c>
       <c r="E5" s="35" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="F5" s="12" t="n">
         <f aca="false">IF(E5="Cut",D5,0)</f>
         <v>0</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>82.99</v>
@@ -12429,25 +12467,25 @@
         <v>995.88</v>
       </c>
       <c r="E6" s="35" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F6" s="12" t="n">
         <f aca="false">IF(E6="Cut",D6,0)</f>
         <v>0</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>26.99</v>
@@ -12457,23 +12495,23 @@
         <v>323.88</v>
       </c>
       <c r="E7" s="35" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="F7" s="12" t="n">
         <f aca="false">IF(E7="Cut",D7,0)</f>
         <v>0</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="H7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>18.99</v>
@@ -12483,25 +12521,25 @@
         <v>227.88</v>
       </c>
       <c r="E8" s="35" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F8" s="12" t="n">
         <f aca="false">IF(E8="Cut",D8,0)</f>
         <v>0</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>12.99</v>
@@ -12511,23 +12549,23 @@
         <v>155.88</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="F9" s="12" t="n">
         <f aca="false">IF(E9="Cut",D9,0)</f>
         <v>0</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="H9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>139</v>
@@ -12537,25 +12575,25 @@
         <v>139</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="F10" s="12" t="n">
         <f aca="false">IF(E10="Cut",D10,0)</f>
         <v>0</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C11" s="6" t="n">
         <v>4.99</v>
@@ -12565,25 +12603,25 @@
         <v>59.88</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F11" s="12" t="n">
         <f aca="false">IF(E11="Cut",D11,0)</f>
         <v>0</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>6.36</v>
@@ -12593,25 +12631,25 @@
         <v>76.32</v>
       </c>
       <c r="E12" s="35" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F12" s="12" t="n">
         <f aca="false">IF(E12="Cut",D12,0)</f>
         <v>0</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C13" s="6" t="n">
         <v>11.99</v>
@@ -12621,25 +12659,25 @@
         <v>143.88</v>
       </c>
       <c r="E13" s="35" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F13" s="12" t="n">
         <f aca="false">IF(E13="Cut",D13,0)</f>
         <v>0</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C14" s="6" t="n">
         <v>8.99</v>
@@ -12649,25 +12687,25 @@
         <v>107.88</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F14" s="12" t="n">
         <f aca="false">IF(E14="Cut",D14,0)</f>
         <v>0</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C15" s="6" t="n">
         <v>25</v>
@@ -12677,25 +12715,25 @@
         <v>300</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F15" s="12" t="n">
         <f aca="false">IF(E15="Cut",D15,0)</f>
         <v>0</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C16" s="6" t="n">
         <v>27.72</v>
@@ -12705,25 +12743,25 @@
         <v>332.64</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F16" s="12" t="n">
         <f aca="false">IF(E16="Cut",D16,0)</f>
         <v>0</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="C17" s="6" t="n">
         <v>99.99</v>
@@ -12733,23 +12771,23 @@
         <v>99.99</v>
       </c>
       <c r="E17" s="35" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F17" s="12" t="n">
         <f aca="false">IF(E17="Cut",D17,0)</f>
         <v>0</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="H17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>400</v>
+        <v>405</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="C18" s="6" t="n">
         <v>150</v>
@@ -12759,23 +12797,23 @@
         <v>150</v>
       </c>
       <c r="E18" s="35" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F18" s="12" t="n">
         <f aca="false">IF(E18="Cut",D18,0)</f>
         <v>0</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>401</v>
+        <v>406</v>
       </c>
       <c r="H18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>402</v>
+        <v>407</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C19" s="6" t="n">
         <v>20.7</v>
@@ -12785,25 +12823,25 @@
         <v>248.4</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="F19" s="12" t="n">
         <f aca="false">IF(E19="Cut",D19,0)</f>
         <v>0</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C20" s="6" t="n">
         <v>10</v>
@@ -12813,25 +12851,25 @@
         <v>120</v>
       </c>
       <c r="E20" s="35" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="F20" s="12" t="n">
         <f aca="false">IF(E20="Cut",D20,0)</f>
         <v>0</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>32.99</v>
@@ -12841,25 +12879,25 @@
         <v>395.88</v>
       </c>
       <c r="E21" s="35" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F21" s="12" t="n">
         <f aca="false">IF(E21="Cut",D21,0)</f>
         <v>0</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C22" s="6" t="n">
         <v>13.94</v>
@@ -12869,25 +12907,25 @@
         <v>167.28</v>
       </c>
       <c r="E22" s="35" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F22" s="12" t="n">
         <f aca="false">IF(E22="Cut",D22,0)</f>
         <v>0</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C23" s="6" t="n">
         <v>20.76</v>
@@ -12897,25 +12935,25 @@
         <v>249.12</v>
       </c>
       <c r="E23" s="35" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F23" s="12" t="n">
         <f aca="false">IF(E23="Cut",D23,0)</f>
         <v>0</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>414</v>
+        <v>419</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C24" s="6" t="n">
         <v>10.63</v>
@@ -12925,23 +12963,23 @@
         <v>127.56</v>
       </c>
       <c r="E24" s="35" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="F24" s="12" t="n">
         <f aca="false">IF(E24="Cut",D24,0)</f>
         <v>0</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="H24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>417</v>
+        <v>422</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C25" s="6" t="n">
         <v>21.25</v>
@@ -12951,23 +12989,23 @@
         <v>255</v>
       </c>
       <c r="E25" s="35" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="F25" s="12" t="n">
         <f aca="false">IF(E25="Cut",D25,0)</f>
         <v>0</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="H25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="C26" s="6" t="n">
         <v>381.44</v>
@@ -12977,25 +13015,25 @@
         <v>381.44</v>
       </c>
       <c r="E26" s="35" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="F26" s="12" t="n">
         <f aca="false">IF(E26="Cut",D26,0)</f>
         <v>0</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>419</v>
+        <v>424</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="C27" s="6" t="n">
         <v>212.49</v>
@@ -13005,25 +13043,25 @@
         <v>212.49</v>
       </c>
       <c r="E27" s="35" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F27" s="12" t="n">
         <f aca="false">IF(E27="Cut",D27,0)</f>
         <v>0</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>423</v>
+        <v>428</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="C28" s="6" t="n">
         <v>114.75</v>
@@ -13033,25 +13071,25 @@
         <v>229.5</v>
       </c>
       <c r="E28" s="35" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F28" s="12" t="n">
         <f aca="false">IF(E28="Cut",D28,0)</f>
         <v>0</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="C29" s="6" t="n">
         <v>548</v>
@@ -13061,25 +13099,25 @@
         <v>548</v>
       </c>
       <c r="E29" s="35" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="F29" s="12" t="n">
         <f aca="false">IF(E29="Cut",D29,0)</f>
         <v>0</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>430</v>
+        <v>435</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>431</v>
+        <v>436</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C30" s="6" t="n">
         <v>32.95</v>
@@ -13089,25 +13127,25 @@
         <v>395.4</v>
       </c>
       <c r="E30" s="35" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F30" s="12" t="n">
         <f aca="false">IF(E30="Cut",D30,0)</f>
         <v>0</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>432</v>
+        <v>437</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>434</v>
+        <v>439</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C31" s="6" t="n">
         <v>115.23</v>
@@ -13117,25 +13155,25 @@
         <v>1382.76</v>
       </c>
       <c r="E31" s="35" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="F31" s="12" t="n">
         <f aca="false">IF(E31="Cut",D31,0)</f>
         <v>0</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>436</v>
+        <v>441</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C32" s="6" t="n">
         <v>25</v>
@@ -13145,22 +13183,22 @@
         <v>300</v>
       </c>
       <c r="E32" s="35" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="F32" s="12" t="n">
         <f aca="false">IF(E32="Cut",D32,0)</f>
         <v>0</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
       <c r="D33" s="17" t="n">
         <f aca="false">SUM(D5:D32)</f>
@@ -13173,7 +13211,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>440</v>
+        <v>445</v>
       </c>
       <c r="D34" s="12" t="n">
         <f aca="false">SUMIF(E5:E32,"Review",D5:D32)</f>
@@ -13182,7 +13220,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>441</v>
+        <v>446</v>
       </c>
     </row>
   </sheetData>
@@ -13210,156 +13248,156 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="36" t="s">
-        <v>443</v>
+        <v>448</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>444</v>
+        <v>449</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="36" t="s">
-        <v>445</v>
+        <v>450</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>446</v>
+        <v>451</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="36" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>448</v>
+        <v>453</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="36" t="s">
-        <v>449</v>
+        <v>454</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>450</v>
+        <v>455</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="36" t="s">
-        <v>451</v>
+        <v>456</v>
       </c>
       <c r="B7" s="37" t="s">
-        <v>452</v>
+        <v>457</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="36" t="s">
-        <v>453</v>
+        <v>458</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>454</v>
+        <v>459</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="36" t="s">
-        <v>455</v>
+        <v>460</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="36" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="36" t="s">
-        <v>459</v>
+        <v>464</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>460</v>
+        <v>465</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="36" t="s">
-        <v>461</v>
+        <v>466</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>462</v>
+        <v>467</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>463</v>
+        <v>468</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="B15" s="37" t="s">
-        <v>465</v>
+        <v>470</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="B16" s="37" t="s">
-        <v>466</v>
+        <v>471</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>467</v>
+        <v>472</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="B18" s="37" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="B19" s="37" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="B20" s="37" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="B21" s="37" t="s">
-        <v>471</v>
+        <v>476</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="B22" s="37" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-10-14 01:40:29
</commit_message>
<xml_diff>
--- a/Dashboards/Areas/💰 Finance/Household Budget 2026-10.xlsx
+++ b/Dashboards/Areas/💰 Finance/Household Budget 2026-10.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="484">
   <si>
     <t xml:space="preserve">Household Budget — October 2026 rebuild</t>
   </si>
@@ -824,6 +824,24 @@
   </si>
   <si>
     <t xml:space="preserve">Set to 5000 to test pulling $5k from SPAXX into JetBlue in Nov-26.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">401(k) catch-up, gross per month (scenario)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age-50 catch-up is $8,000 in 2026. $667 = full-year pace; $889 = the full $8k squeezed into Apr–Dec 2027. 0 = not doing it. Phase 1 says no new investing until cards are cleared.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catch-up starts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First month after the cards clear.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Federal tax shield on catch-up (0% if Roth)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre-tax: ~32% federal. MA does not exempt 401(k) deferrals (my read — confirm with your CPA). Roth catch-up: enter 0%.</t>
   </si>
   <si>
     <t xml:space="preserve">Bonus lump lands in month</t>
@@ -4631,7 +4649,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:W92"/>
+  <dimension ref="A1:W95"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
@@ -4685,7 +4703,7 @@
         <v>195</v>
       </c>
       <c r="G5" s="29" t="n">
-        <f aca="false">IFERROR(INDEX(A45:A92,MATCH(1,Q45:Q92,0)),"after Oct-30")</f>
+        <f aca="false">IFERROR(INDEX(A48:A95,MATCH(1,Q48:Q95,0)),"after Oct-30")</f>
         <v>46447</v>
       </c>
     </row>
@@ -4703,7 +4721,7 @@
         <v>198</v>
       </c>
       <c r="G6" s="29" t="n">
-        <f aca="false">IFERROR(INDEX(A45:A92,MATCH(1,R45:R92,0)),"after Oct-30")</f>
+        <f aca="false">IFERROR(INDEX(A48:A95,MATCH(1,R48:R95,0)),"after Oct-30")</f>
         <v>46447</v>
       </c>
     </row>
@@ -4721,7 +4739,7 @@
         <v>200</v>
       </c>
       <c r="G7" s="29" t="n">
-        <f aca="false">IFERROR(INDEX(A45:A92,MATCH(1,S45:S92,0)),"after Oct-30")</f>
+        <f aca="false">IFERROR(INDEX(A48:A95,MATCH(1,S48:S95,0)),"after Oct-30")</f>
         <v>46447</v>
       </c>
     </row>
@@ -4739,7 +4757,7 @@
         <v>202</v>
       </c>
       <c r="G8" s="29" t="n">
-        <f aca="false">IFERROR(INDEX(A45:A92,MATCH(1,T45:T92,0)),"after Oct-30")</f>
+        <f aca="false">IFERROR(INDEX(A48:A95,MATCH(1,T48:T95,0)),"after Oct-30")</f>
         <v>46447</v>
       </c>
     </row>
@@ -4757,7 +4775,7 @@
         <v>205</v>
       </c>
       <c r="G9" s="29" t="n">
-        <f aca="false">IFERROR(INDEX(A45:A92,MATCH(1,U45:U92,0)),"after Oct-30")</f>
+        <f aca="false">IFERROR(INDEX(A48:A95,MATCH(1,U48:U95,0)),"after Oct-30")</f>
         <v>46874</v>
       </c>
     </row>
@@ -4775,7 +4793,7 @@
         <v>208</v>
       </c>
       <c r="G10" s="9" t="n">
-        <f aca="false">SUM(F45:F92)+SUM(J45:J92)</f>
+        <f aca="false">SUM(F48:F95)+SUM(J48:J95)</f>
         <v>1442.47513468667</v>
       </c>
     </row>
@@ -5112,394 +5130,148 @@
       <c r="A39" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="B39" s="26" t="n">
-        <v>46447</v>
-      </c>
-      <c r="C39" s="2"/>
+      <c r="B39" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>267</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B40" s="26" t="n">
-        <v>47119</v>
+        <v>46478</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>269</v>
-      </c>
-      <c r="B41" s="21" t="n">
+        <v>270</v>
+      </c>
+      <c r="B41" s="31" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="B42" s="26" t="n">
+        <v>46447</v>
+      </c>
+      <c r="C42" s="2"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="B43" s="26" t="n">
+        <v>47119</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="B44" s="21" t="n">
         <f aca="false">Budget!F16</f>
         <v>342</v>
       </c>
-      <c r="C41" s="2" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="10" t="s">
-        <v>271</v>
-      </c>
-      <c r="B44" s="10" t="s">
-        <v>272</v>
-      </c>
-      <c r="C44" s="10" t="s">
-        <v>273</v>
-      </c>
-      <c r="D44" s="10" t="s">
-        <v>274</v>
-      </c>
-      <c r="E44" s="10" t="s">
-        <v>275</v>
-      </c>
-      <c r="F44" s="10" t="s">
+      <c r="C44" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="G44" s="10" t="s">
+    </row>
+    <row r="47" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="10" t="s">
         <v>277</v>
       </c>
-      <c r="H44" s="10" t="s">
+      <c r="B47" s="10" t="s">
         <v>278</v>
       </c>
-      <c r="I44" s="10" t="s">
+      <c r="C47" s="10" t="s">
         <v>279</v>
       </c>
-      <c r="J44" s="10" t="s">
+      <c r="D47" s="10" t="s">
         <v>280</v>
       </c>
-      <c r="K44" s="10" t="s">
+      <c r="E47" s="10" t="s">
         <v>281</v>
       </c>
-      <c r="L44" s="10" t="s">
+      <c r="F47" s="10" t="s">
         <v>282</v>
       </c>
-      <c r="M44" s="10" t="s">
+      <c r="G47" s="10" t="s">
         <v>283</v>
       </c>
-      <c r="N44" s="10" t="s">
+      <c r="H47" s="10" t="s">
         <v>284</v>
       </c>
-      <c r="O44" s="10" t="s">
+      <c r="I47" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="P44" s="10" t="s">
+      <c r="J47" s="10" t="s">
         <v>286</v>
       </c>
-      <c r="Q44" s="10" t="s">
+      <c r="K47" s="10" t="s">
         <v>287</v>
       </c>
-      <c r="R44" s="10" t="s">
+      <c r="L47" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="S44" s="10" t="s">
+      <c r="M47" s="10" t="s">
         <v>289</v>
       </c>
-      <c r="T44" s="10" t="s">
+      <c r="N47" s="10" t="s">
         <v>290</v>
       </c>
-      <c r="U44" s="10" t="s">
+      <c r="O47" s="10" t="s">
         <v>291</v>
       </c>
-      <c r="V44" s="10" t="s">
+      <c r="P47" s="10" t="s">
         <v>292</v>
       </c>
-      <c r="W44" s="10" t="s">
+      <c r="Q47" s="10" t="s">
         <v>293</v>
       </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="34" t="n">
-        <v>46327</v>
-      </c>
-      <c r="B45" s="21" t="n">
-        <f aca="false">IF(A45&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A45&gt;$B$40,$B$41,0)+IF(A45&gt;=$B$35,$B$37,0)+$B$32</f>
-        <v>977.318333333335</v>
-      </c>
-      <c r="C45" s="12" t="n">
-        <f aca="false">IF(A45=$B$39,$B$26-$B$29,0)-IF(A45=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A45=$B$35,$B$37*$B$36,0)+$B$38</f>
-        <v>0</v>
-      </c>
-      <c r="D45" s="12" t="n">
-        <f aca="false">B45+C45</f>
-        <v>977.318333333335</v>
-      </c>
-      <c r="E45" s="12" t="n">
-        <f aca="false">$B$5</f>
-        <v>9800.78</v>
-      </c>
-      <c r="F45" s="12" t="n">
-        <f aca="false">E45*$B$6/12</f>
-        <v>242.895997666667</v>
-      </c>
-      <c r="G45" s="12" t="n">
-        <f aca="false">MIN(E45+F45,MAX(D45-K45,0))</f>
-        <v>846.050479333335</v>
-      </c>
-      <c r="H45" s="12" t="n">
-        <f aca="false">E45+F45-G45</f>
-        <v>9197.62551833333</v>
-      </c>
-      <c r="I45" s="12" t="n">
-        <f aca="false">$B$7</f>
-        <v>5341.52</v>
-      </c>
-      <c r="J45" s="12" t="n">
-        <f aca="false">I45*$B$8/12</f>
-        <v>77.852654</v>
-      </c>
-      <c r="K45" s="12" t="n">
-        <f aca="false">MIN(I45+J45,J45+$B$9*I45)</f>
-        <v>131.267854</v>
-      </c>
-      <c r="L45" s="12" t="n">
-        <f aca="false">MIN(I45+J45,MAX(D45-G45,0))</f>
-        <v>131.267854</v>
-      </c>
-      <c r="M45" s="12" t="n">
-        <f aca="false">I45+J45-L45</f>
-        <v>5288.1048</v>
-      </c>
-      <c r="N45" s="12" t="n">
-        <f aca="false">$B$10-$B$38</f>
-        <v>12081</v>
-      </c>
-      <c r="O45" s="12" t="n">
-        <f aca="false">MIN(D45-G45-L45,MAX($B$15-$B$18-N45,0))</f>
-        <v>0</v>
-      </c>
-      <c r="P45" s="12" t="n">
-        <f aca="false">N45+O45</f>
-        <v>12081</v>
-      </c>
-      <c r="Q45" s="5" t="n">
-        <f aca="false">IF(H45&lt;=0.005,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="R45" s="5" t="n">
-        <f aca="false">IF(M45&lt;=0.005,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="S45" s="5" t="n">
-        <f aca="false">IF(AND(Q45=1,R45=1),1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="T45" s="5" t="n">
-        <f aca="false">IF(P45&gt;=$B$20,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="U45" s="5" t="n">
-        <f aca="false">IF(P45+$B$18&gt;=$B$15-0.5,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="V45" s="12" t="n">
-        <f aca="false">MAX(D45-G45-L45,0)-MAX(O45,0)</f>
-        <v>0</v>
-      </c>
-      <c r="W45" s="12" t="n">
-        <f aca="false">P45+$B$18</f>
-        <v>28341.75</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="34" t="n">
-        <v>46357</v>
-      </c>
-      <c r="B46" s="21" t="n">
-        <f aca="false">IF(A46&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A46&gt;$B$40,$B$41,0)+IF(A46&gt;=$B$35,$B$37,0)+$B$32</f>
-        <v>977.318333333335</v>
-      </c>
-      <c r="C46" s="12" t="n">
-        <f aca="false">IF(A46=$B$39,$B$26-$B$29,0)-IF(A46=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A46=$B$35,$B$37*$B$36,0)+0</f>
-        <v>0</v>
-      </c>
-      <c r="D46" s="12" t="n">
-        <f aca="false">B46+C46</f>
-        <v>977.318333333335</v>
-      </c>
-      <c r="E46" s="12" t="n">
-        <f aca="false">H45</f>
-        <v>9197.62551833333</v>
-      </c>
-      <c r="F46" s="12" t="n">
-        <f aca="false">E46*$B$6/12</f>
-        <v>227.947819096028</v>
-      </c>
-      <c r="G46" s="12" t="n">
-        <f aca="false">MIN(E46+F46,MAX(D46-K46,0))</f>
-        <v>847.363157873335</v>
-      </c>
-      <c r="H46" s="12" t="n">
-        <f aca="false">E46+F46-G46</f>
-        <v>8578.21017955603</v>
-      </c>
-      <c r="I46" s="12" t="n">
-        <f aca="false">M45</f>
-        <v>5288.1048</v>
-      </c>
-      <c r="J46" s="12" t="n">
-        <f aca="false">I46*$B$8/12</f>
-        <v>77.07412746</v>
-      </c>
-      <c r="K46" s="12" t="n">
-        <f aca="false">MIN(I46+J46,J46+$B$9*I46)</f>
-        <v>129.95517546</v>
-      </c>
-      <c r="L46" s="12" t="n">
-        <f aca="false">MIN(I46+J46,MAX(D46-G46,0))</f>
-        <v>129.95517546</v>
-      </c>
-      <c r="M46" s="12" t="n">
-        <f aca="false">I46+J46-L46</f>
-        <v>5235.223752</v>
-      </c>
-      <c r="N46" s="12" t="n">
-        <f aca="false">P45</f>
-        <v>12081</v>
-      </c>
-      <c r="O46" s="12" t="n">
-        <f aca="false">MIN(D46-G46-L46,MAX($B$15-$B$18-N46,0))</f>
-        <v>0</v>
-      </c>
-      <c r="P46" s="12" t="n">
-        <f aca="false">N46+O46</f>
-        <v>12081</v>
-      </c>
-      <c r="Q46" s="5" t="n">
-        <f aca="false">IF(H46&lt;=0.005,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="R46" s="5" t="n">
-        <f aca="false">IF(M46&lt;=0.005,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="S46" s="5" t="n">
-        <f aca="false">IF(AND(Q46=1,R46=1),1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="T46" s="5" t="n">
-        <f aca="false">IF(P46&gt;=$B$20,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="U46" s="5" t="n">
-        <f aca="false">IF(P46+$B$18&gt;=$B$15-0.5,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="V46" s="12" t="n">
-        <f aca="false">MAX(D46-G46-L46,0)-MAX(O46,0)</f>
-        <v>0</v>
-      </c>
-      <c r="W46" s="12" t="n">
-        <f aca="false">P46+$B$18</f>
-        <v>28341.75</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="34" t="n">
-        <v>46388</v>
-      </c>
-      <c r="B47" s="21" t="n">
-        <f aca="false">IF(A47&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A47&gt;$B$40,$B$41,0)+IF(A47&gt;=$B$35,$B$37,0)+$B$32</f>
-        <v>977.318333333335</v>
-      </c>
-      <c r="C47" s="12" t="n">
-        <f aca="false">IF(A47=$B$39,$B$26-$B$29,0)-IF(A47=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A47=$B$35,$B$37*$B$36,0)+0</f>
-        <v>0</v>
-      </c>
-      <c r="D47" s="12" t="n">
-        <f aca="false">B47+C47</f>
-        <v>977.318333333335</v>
-      </c>
-      <c r="E47" s="12" t="n">
-        <f aca="false">H46</f>
-        <v>8578.21017955603</v>
-      </c>
-      <c r="F47" s="12" t="n">
-        <f aca="false">E47*$B$6/12</f>
-        <v>212.59664228333</v>
-      </c>
-      <c r="G47" s="12" t="n">
-        <f aca="false">MIN(E47+F47,MAX(D47-K47,0))</f>
-        <v>848.662709627935</v>
-      </c>
-      <c r="H47" s="12" t="n">
-        <f aca="false">E47+F47-G47</f>
-        <v>7942.14411221142</v>
-      </c>
-      <c r="I47" s="12" t="n">
-        <f aca="false">M46</f>
-        <v>5235.223752</v>
-      </c>
-      <c r="J47" s="12" t="n">
-        <f aca="false">I47*$B$8/12</f>
-        <v>76.3033861854</v>
-      </c>
-      <c r="K47" s="12" t="n">
-        <f aca="false">MIN(I47+J47,J47+$B$9*I47)</f>
-        <v>128.6556237054</v>
-      </c>
-      <c r="L47" s="12" t="n">
-        <f aca="false">MIN(I47+J47,MAX(D47-G47,0))</f>
-        <v>128.6556237054</v>
-      </c>
-      <c r="M47" s="12" t="n">
-        <f aca="false">I47+J47-L47</f>
-        <v>5182.87151448</v>
-      </c>
-      <c r="N47" s="12" t="n">
-        <f aca="false">P46</f>
-        <v>12081</v>
-      </c>
-      <c r="O47" s="12" t="n">
-        <f aca="false">MIN(D47-G47-L47,MAX($B$15-$B$18-N47,0))</f>
-        <v>0</v>
-      </c>
-      <c r="P47" s="12" t="n">
-        <f aca="false">N47+O47</f>
-        <v>12081</v>
-      </c>
-      <c r="Q47" s="5" t="n">
-        <f aca="false">IF(H47&lt;=0.005,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="R47" s="5" t="n">
-        <f aca="false">IF(M47&lt;=0.005,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="S47" s="5" t="n">
-        <f aca="false">IF(AND(Q47=1,R47=1),1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="T47" s="5" t="n">
-        <f aca="false">IF(P47&gt;=$B$20,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="U47" s="5" t="n">
-        <f aca="false">IF(P47+$B$18&gt;=$B$15-0.5,1,0)</f>
-        <v>0</v>
-      </c>
-      <c r="V47" s="12" t="n">
-        <f aca="false">MAX(D47-G47-L47,0)-MAX(O47,0)</f>
-        <v>0</v>
-      </c>
-      <c r="W47" s="12" t="n">
-        <f aca="false">P47+$B$18</f>
-        <v>28341.75</v>
+      <c r="R47" s="10" t="s">
+        <v>294</v>
+      </c>
+      <c r="S47" s="10" t="s">
+        <v>295</v>
+      </c>
+      <c r="T47" s="10" t="s">
+        <v>296</v>
+      </c>
+      <c r="U47" s="10" t="s">
+        <v>297</v>
+      </c>
+      <c r="V47" s="10" t="s">
+        <v>298</v>
+      </c>
+      <c r="W47" s="10" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="34" t="n">
-        <v>46419</v>
+        <v>46327</v>
       </c>
       <c r="B48" s="21" t="n">
-        <f aca="false">IF(A48&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A48&gt;$B$40,$B$41,0)+IF(A48&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A48&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A48&gt;$B$43,$B$44,0)+IF(A48&gt;=$B$35,$B$37,0)+$B$32-IF(A48&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>977.318333333335</v>
       </c>
       <c r="C48" s="12" t="n">
-        <f aca="false">IF(A48=$B$39,$B$26-$B$29,0)-IF(A48=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A48=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A48=$B$42,$B$26-$B$29,0)-IF(A48=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A48=$B$35,$B$37*$B$36,0)+$B$38</f>
         <v>0</v>
       </c>
       <c r="D48" s="12" t="n">
@@ -5507,43 +5279,43 @@
         <v>977.318333333335</v>
       </c>
       <c r="E48" s="12" t="n">
-        <f aca="false">H47</f>
-        <v>7942.14411221142</v>
+        <f aca="false">$B$5</f>
+        <v>9800.78</v>
       </c>
       <c r="F48" s="12" t="n">
         <f aca="false">E48*$B$6/12</f>
-        <v>196.832804914306</v>
+        <v>242.895997666667</v>
       </c>
       <c r="G48" s="12" t="n">
         <f aca="false">MIN(E48+F48,MAX(D48-K48,0))</f>
-        <v>849.949265864989</v>
+        <v>846.050479333335</v>
       </c>
       <c r="H48" s="12" t="n">
         <f aca="false">E48+F48-G48</f>
-        <v>7289.02765126074</v>
+        <v>9197.62551833333</v>
       </c>
       <c r="I48" s="12" t="n">
-        <f aca="false">M47</f>
-        <v>5182.87151448</v>
+        <f aca="false">$B$7</f>
+        <v>5341.52</v>
       </c>
       <c r="J48" s="12" t="n">
         <f aca="false">I48*$B$8/12</f>
-        <v>75.540352323546</v>
+        <v>77.852654</v>
       </c>
       <c r="K48" s="12" t="n">
         <f aca="false">MIN(I48+J48,J48+$B$9*I48)</f>
-        <v>127.369067468346</v>
+        <v>131.267854</v>
       </c>
       <c r="L48" s="12" t="n">
         <f aca="false">MIN(I48+J48,MAX(D48-G48,0))</f>
-        <v>127.369067468346</v>
+        <v>131.267854</v>
       </c>
       <c r="M48" s="12" t="n">
         <f aca="false">I48+J48-L48</f>
-        <v>5131.0427993352</v>
+        <v>5288.1048</v>
       </c>
       <c r="N48" s="12" t="n">
-        <f aca="false">P47</f>
+        <f aca="false">$B$10-$B$38</f>
         <v>12081</v>
       </c>
       <c r="O48" s="12" t="n">
@@ -5585,55 +5357,55 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="34" t="n">
-        <v>46447</v>
+        <v>46357</v>
       </c>
       <c r="B49" s="21" t="n">
-        <f aca="false">IF(A49&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A49&gt;$B$40,$B$41,0)+IF(A49&gt;=$B$35,$B$37,0)+$B$32</f>
-        <v>2569.09333333334</v>
+        <f aca="false">IF(A49&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A49&gt;$B$43,$B$44,0)+IF(A49&gt;=$B$35,$B$37,0)+$B$32-IF(A49&gt;=$B$40,$B$39*(1-$B$41),0)</f>
+        <v>977.318333333335</v>
       </c>
       <c r="C49" s="12" t="n">
-        <f aca="false">IF(A49=$B$39,$B$26-$B$29,0)-IF(A49=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A49=$B$35,$B$37*$B$36,0)+0</f>
-        <v>51581.8416666667</v>
+        <f aca="false">IF(A49=$B$42,$B$26-$B$29,0)-IF(A49=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A49=$B$35,$B$37*$B$36,0)+0</f>
+        <v>0</v>
       </c>
       <c r="D49" s="12" t="n">
         <f aca="false">B49+C49</f>
-        <v>54150.935</v>
+        <v>977.318333333335</v>
       </c>
       <c r="E49" s="12" t="n">
         <f aca="false">H48</f>
-        <v>7289.02765126074</v>
+        <v>9197.62551833333</v>
       </c>
       <c r="F49" s="12" t="n">
         <f aca="false">E49*$B$6/12</f>
-        <v>180.646401957079</v>
+        <v>227.947819096028</v>
       </c>
       <c r="G49" s="12" t="n">
         <f aca="false">MIN(E49+F49,MAX(D49-K49,0))</f>
-        <v>7469.67405321782</v>
+        <v>847.363157873335</v>
       </c>
       <c r="H49" s="12" t="n">
         <f aca="false">E49+F49-G49</f>
-        <v>0</v>
+        <v>8578.21017955603</v>
       </c>
       <c r="I49" s="12" t="n">
         <f aca="false">M48</f>
-        <v>5131.0427993352</v>
+        <v>5288.1048</v>
       </c>
       <c r="J49" s="12" t="n">
         <f aca="false">I49*$B$8/12</f>
-        <v>74.7849488003106</v>
+        <v>77.07412746</v>
       </c>
       <c r="K49" s="12" t="n">
         <f aca="false">MIN(I49+J49,J49+$B$9*I49)</f>
-        <v>126.095376793663</v>
+        <v>129.95517546</v>
       </c>
       <c r="L49" s="12" t="n">
         <f aca="false">MIN(I49+J49,MAX(D49-G49,0))</f>
-        <v>5205.82774813551</v>
+        <v>129.95517546</v>
       </c>
       <c r="M49" s="12" t="n">
         <f aca="false">I49+J49-L49</f>
-        <v>0</v>
+        <v>5235.223752</v>
       </c>
       <c r="N49" s="12" t="n">
         <f aca="false">P48</f>
@@ -5641,27 +5413,27 @@
       </c>
       <c r="O49" s="12" t="n">
         <f aca="false">MIN(D49-G49-L49,MAX($B$15-$B$18-N49,0))</f>
-        <v>41475.4331986467</v>
+        <v>0</v>
       </c>
       <c r="P49" s="12" t="n">
         <f aca="false">N49+O49</f>
-        <v>53556.4331986467</v>
+        <v>12081</v>
       </c>
       <c r="Q49" s="5" t="n">
         <f aca="false">IF(H49&lt;=0.005,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R49" s="5" t="n">
         <f aca="false">IF(M49&lt;=0.005,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S49" s="5" t="n">
         <f aca="false">IF(AND(Q49=1,R49=1),1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T49" s="5" t="n">
         <f aca="false">IF(P49&gt;=$B$20,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U49" s="5" t="n">
         <f aca="false">IF(P49+$B$18&gt;=$B$15-0.5,1,0)</f>
@@ -5673,88 +5445,88 @@
       </c>
       <c r="W49" s="12" t="n">
         <f aca="false">P49+$B$18</f>
-        <v>69817.1831986467</v>
+        <v>28341.75</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="34" t="n">
-        <v>46478</v>
+        <v>46388</v>
       </c>
       <c r="B50" s="21" t="n">
-        <f aca="false">IF(A50&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A50&gt;$B$40,$B$41,0)+IF(A50&gt;=$B$35,$B$37,0)+$B$32</f>
-        <v>2569.09333333334</v>
+        <f aca="false">IF(A50&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A50&gt;$B$43,$B$44,0)+IF(A50&gt;=$B$35,$B$37,0)+$B$32-IF(A50&gt;=$B$40,$B$39*(1-$B$41),0)</f>
+        <v>977.318333333335</v>
       </c>
       <c r="C50" s="12" t="n">
-        <f aca="false">IF(A50=$B$39,$B$26-$B$29,0)-IF(A50=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A50=$B$35,$B$37*$B$36,0)+0</f>
-        <v>-3983.25</v>
+        <f aca="false">IF(A50=$B$42,$B$26-$B$29,0)-IF(A50=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A50=$B$35,$B$37*$B$36,0)+0</f>
+        <v>0</v>
       </c>
       <c r="D50" s="12" t="n">
         <f aca="false">B50+C50</f>
-        <v>-1414.15666666667</v>
+        <v>977.318333333335</v>
       </c>
       <c r="E50" s="12" t="n">
         <f aca="false">H49</f>
-        <v>0</v>
+        <v>8578.21017955603</v>
       </c>
       <c r="F50" s="12" t="n">
         <f aca="false">E50*$B$6/12</f>
-        <v>0</v>
+        <v>212.59664228333</v>
       </c>
       <c r="G50" s="12" t="n">
         <f aca="false">MIN(E50+F50,MAX(D50-K50,0))</f>
-        <v>0</v>
+        <v>848.662709627935</v>
       </c>
       <c r="H50" s="12" t="n">
         <f aca="false">E50+F50-G50</f>
-        <v>0</v>
+        <v>7942.14411221142</v>
       </c>
       <c r="I50" s="12" t="n">
         <f aca="false">M49</f>
-        <v>0</v>
+        <v>5235.223752</v>
       </c>
       <c r="J50" s="12" t="n">
         <f aca="false">I50*$B$8/12</f>
-        <v>0</v>
+        <v>76.3033861854</v>
       </c>
       <c r="K50" s="12" t="n">
         <f aca="false">MIN(I50+J50,J50+$B$9*I50)</f>
-        <v>0</v>
+        <v>128.6556237054</v>
       </c>
       <c r="L50" s="12" t="n">
         <f aca="false">MIN(I50+J50,MAX(D50-G50,0))</f>
-        <v>0</v>
+        <v>128.6556237054</v>
       </c>
       <c r="M50" s="12" t="n">
         <f aca="false">I50+J50-L50</f>
-        <v>0</v>
+        <v>5182.87151448</v>
       </c>
       <c r="N50" s="12" t="n">
         <f aca="false">P49</f>
-        <v>53556.4331986467</v>
+        <v>12081</v>
       </c>
       <c r="O50" s="12" t="n">
         <f aca="false">MIN(D50-G50-L50,MAX($B$15-$B$18-N50,0))</f>
-        <v>-1414.15666666667</v>
+        <v>0</v>
       </c>
       <c r="P50" s="12" t="n">
         <f aca="false">N50+O50</f>
-        <v>52142.27653198</v>
+        <v>12081</v>
       </c>
       <c r="Q50" s="5" t="n">
         <f aca="false">IF(H50&lt;=0.005,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R50" s="5" t="n">
         <f aca="false">IF(M50&lt;=0.005,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S50" s="5" t="n">
         <f aca="false">IF(AND(Q50=1,R50=1),1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T50" s="5" t="n">
         <f aca="false">IF(P50&gt;=$B$20,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U50" s="5" t="n">
         <f aca="false">IF(P50+$B$18&gt;=$B$15-0.5,1,0)</f>
@@ -5766,88 +5538,88 @@
       </c>
       <c r="W50" s="12" t="n">
         <f aca="false">P50+$B$18</f>
-        <v>68403.02653198</v>
+        <v>28341.75</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="34" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="B51" s="21" t="n">
-        <f aca="false">IF(A51&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A51&gt;$B$40,$B$41,0)+IF(A51&gt;=$B$35,$B$37,0)+$B$32</f>
-        <v>2569.09333333334</v>
+        <f aca="false">IF(A51&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A51&gt;$B$43,$B$44,0)+IF(A51&gt;=$B$35,$B$37,0)+$B$32-IF(A51&gt;=$B$40,$B$39*(1-$B$41),0)</f>
+        <v>977.318333333335</v>
       </c>
       <c r="C51" s="12" t="n">
-        <f aca="false">IF(A51=$B$39,$B$26-$B$29,0)-IF(A51=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A51=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A51=$B$42,$B$26-$B$29,0)-IF(A51=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A51=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D51" s="12" t="n">
         <f aca="false">B51+C51</f>
-        <v>2569.09333333334</v>
+        <v>977.318333333335</v>
       </c>
       <c r="E51" s="12" t="n">
         <f aca="false">H50</f>
-        <v>0</v>
+        <v>7942.14411221142</v>
       </c>
       <c r="F51" s="12" t="n">
         <f aca="false">E51*$B$6/12</f>
-        <v>0</v>
+        <v>196.832804914306</v>
       </c>
       <c r="G51" s="12" t="n">
         <f aca="false">MIN(E51+F51,MAX(D51-K51,0))</f>
-        <v>0</v>
+        <v>849.949265864989</v>
       </c>
       <c r="H51" s="12" t="n">
         <f aca="false">E51+F51-G51</f>
-        <v>0</v>
+        <v>7289.02765126074</v>
       </c>
       <c r="I51" s="12" t="n">
         <f aca="false">M50</f>
-        <v>0</v>
+        <v>5182.87151448</v>
       </c>
       <c r="J51" s="12" t="n">
         <f aca="false">I51*$B$8/12</f>
-        <v>0</v>
+        <v>75.540352323546</v>
       </c>
       <c r="K51" s="12" t="n">
         <f aca="false">MIN(I51+J51,J51+$B$9*I51)</f>
-        <v>0</v>
+        <v>127.369067468346</v>
       </c>
       <c r="L51" s="12" t="n">
         <f aca="false">MIN(I51+J51,MAX(D51-G51,0))</f>
-        <v>0</v>
+        <v>127.369067468346</v>
       </c>
       <c r="M51" s="12" t="n">
         <f aca="false">I51+J51-L51</f>
-        <v>0</v>
+        <v>5131.0427993352</v>
       </c>
       <c r="N51" s="12" t="n">
         <f aca="false">P50</f>
-        <v>52142.27653198</v>
+        <v>12081</v>
       </c>
       <c r="O51" s="12" t="n">
         <f aca="false">MIN(D51-G51-L51,MAX($B$15-$B$18-N51,0))</f>
-        <v>2569.09333333334</v>
+        <v>0</v>
       </c>
       <c r="P51" s="12" t="n">
         <f aca="false">N51+O51</f>
-        <v>54711.3698653134</v>
+        <v>12081</v>
       </c>
       <c r="Q51" s="5" t="n">
         <f aca="false">IF(H51&lt;=0.005,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R51" s="5" t="n">
         <f aca="false">IF(M51&lt;=0.005,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S51" s="5" t="n">
         <f aca="false">IF(AND(Q51=1,R51=1),1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T51" s="5" t="n">
         <f aca="false">IF(P51&gt;=$B$20,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U51" s="5" t="n">
         <f aca="false">IF(P51+$B$18&gt;=$B$15-0.5,1,0)</f>
@@ -5859,36 +5631,36 @@
       </c>
       <c r="W51" s="12" t="n">
         <f aca="false">P51+$B$18</f>
-        <v>70972.1198653134</v>
+        <v>28341.75</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="34" t="n">
-        <v>46539</v>
+        <v>46447</v>
       </c>
       <c r="B52" s="21" t="n">
-        <f aca="false">IF(A52&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A52&gt;$B$40,$B$41,0)+IF(A52&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A52&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A52&gt;$B$43,$B$44,0)+IF(A52&gt;=$B$35,$B$37,0)+$B$32-IF(A52&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C52" s="12" t="n">
-        <f aca="false">IF(A52=$B$39,$B$26-$B$29,0)-IF(A52=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A52=$B$35,$B$37*$B$36,0)+0</f>
-        <v>0</v>
+        <f aca="false">IF(A52=$B$42,$B$26-$B$29,0)-IF(A52=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A52=$B$35,$B$37*$B$36,0)+0</f>
+        <v>51581.8416666667</v>
       </c>
       <c r="D52" s="12" t="n">
         <f aca="false">B52+C52</f>
-        <v>2569.09333333334</v>
+        <v>54150.935</v>
       </c>
       <c r="E52" s="12" t="n">
         <f aca="false">H51</f>
-        <v>0</v>
+        <v>7289.02765126074</v>
       </c>
       <c r="F52" s="12" t="n">
         <f aca="false">E52*$B$6/12</f>
-        <v>0</v>
+        <v>180.646401957079</v>
       </c>
       <c r="G52" s="12" t="n">
         <f aca="false">MIN(E52+F52,MAX(D52-K52,0))</f>
-        <v>0</v>
+        <v>7469.67405321782</v>
       </c>
       <c r="H52" s="12" t="n">
         <f aca="false">E52+F52-G52</f>
@@ -5896,19 +5668,19 @@
       </c>
       <c r="I52" s="12" t="n">
         <f aca="false">M51</f>
-        <v>0</v>
+        <v>5131.0427993352</v>
       </c>
       <c r="J52" s="12" t="n">
         <f aca="false">I52*$B$8/12</f>
-        <v>0</v>
+        <v>74.7849488003106</v>
       </c>
       <c r="K52" s="12" t="n">
         <f aca="false">MIN(I52+J52,J52+$B$9*I52)</f>
-        <v>0</v>
+        <v>126.095376793663</v>
       </c>
       <c r="L52" s="12" t="n">
         <f aca="false">MIN(I52+J52,MAX(D52-G52,0))</f>
-        <v>0</v>
+        <v>5205.82774813551</v>
       </c>
       <c r="M52" s="12" t="n">
         <f aca="false">I52+J52-L52</f>
@@ -5916,15 +5688,15 @@
       </c>
       <c r="N52" s="12" t="n">
         <f aca="false">P51</f>
-        <v>54711.3698653134</v>
+        <v>12081</v>
       </c>
       <c r="O52" s="12" t="n">
         <f aca="false">MIN(D52-G52-L52,MAX($B$15-$B$18-N52,0))</f>
-        <v>2569.09333333334</v>
+        <v>41475.4331986467</v>
       </c>
       <c r="P52" s="12" t="n">
         <f aca="false">N52+O52</f>
-        <v>57280.4631986467</v>
+        <v>53556.4331986467</v>
       </c>
       <c r="Q52" s="5" t="n">
         <f aca="false">IF(H52&lt;=0.005,1,0)</f>
@@ -5952,24 +5724,24 @@
       </c>
       <c r="W52" s="12" t="n">
         <f aca="false">P52+$B$18</f>
-        <v>73541.2131986467</v>
+        <v>69817.1831986467</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="34" t="n">
-        <v>46569</v>
+        <v>46478</v>
       </c>
       <c r="B53" s="21" t="n">
-        <f aca="false">IF(A53&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A53&gt;$B$40,$B$41,0)+IF(A53&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A53&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A53&gt;$B$43,$B$44,0)+IF(A53&gt;=$B$35,$B$37,0)+$B$32-IF(A53&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C53" s="12" t="n">
-        <f aca="false">IF(A53=$B$39,$B$26-$B$29,0)-IF(A53=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A53=$B$35,$B$37*$B$36,0)+0</f>
-        <v>0</v>
+        <f aca="false">IF(A53=$B$42,$B$26-$B$29,0)-IF(A53=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A53=$B$35,$B$37*$B$36,0)+0</f>
+        <v>-3983.25</v>
       </c>
       <c r="D53" s="12" t="n">
         <f aca="false">B53+C53</f>
-        <v>2569.09333333334</v>
+        <v>-1414.15666666667</v>
       </c>
       <c r="E53" s="12" t="n">
         <f aca="false">H52</f>
@@ -6009,15 +5781,15 @@
       </c>
       <c r="N53" s="12" t="n">
         <f aca="false">P52</f>
-        <v>57280.4631986467</v>
+        <v>53556.4331986467</v>
       </c>
       <c r="O53" s="12" t="n">
         <f aca="false">MIN(D53-G53-L53,MAX($B$15-$B$18-N53,0))</f>
-        <v>2569.09333333334</v>
+        <v>-1414.15666666667</v>
       </c>
       <c r="P53" s="12" t="n">
         <f aca="false">N53+O53</f>
-        <v>59849.55653198</v>
+        <v>52142.27653198</v>
       </c>
       <c r="Q53" s="5" t="n">
         <f aca="false">IF(H53&lt;=0.005,1,0)</f>
@@ -6045,19 +5817,19 @@
       </c>
       <c r="W53" s="12" t="n">
         <f aca="false">P53+$B$18</f>
-        <v>76110.30653198</v>
+        <v>68403.02653198</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="34" t="n">
-        <v>46600</v>
+        <v>46508</v>
       </c>
       <c r="B54" s="21" t="n">
-        <f aca="false">IF(A54&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A54&gt;$B$40,$B$41,0)+IF(A54&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A54&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A54&gt;$B$43,$B$44,0)+IF(A54&gt;=$B$35,$B$37,0)+$B$32-IF(A54&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C54" s="12" t="n">
-        <f aca="false">IF(A54=$B$39,$B$26-$B$29,0)-IF(A54=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A54=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A54=$B$42,$B$26-$B$29,0)-IF(A54=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A54=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D54" s="12" t="n">
@@ -6102,7 +5874,7 @@
       </c>
       <c r="N54" s="12" t="n">
         <f aca="false">P53</f>
-        <v>59849.55653198</v>
+        <v>52142.27653198</v>
       </c>
       <c r="O54" s="12" t="n">
         <f aca="false">MIN(D54-G54-L54,MAX($B$15-$B$18-N54,0))</f>
@@ -6110,7 +5882,7 @@
       </c>
       <c r="P54" s="12" t="n">
         <f aca="false">N54+O54</f>
-        <v>62418.6498653134</v>
+        <v>54711.3698653134</v>
       </c>
       <c r="Q54" s="5" t="n">
         <f aca="false">IF(H54&lt;=0.005,1,0)</f>
@@ -6138,19 +5910,19 @@
       </c>
       <c r="W54" s="12" t="n">
         <f aca="false">P54+$B$18</f>
-        <v>78679.3998653134</v>
+        <v>70972.1198653134</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="34" t="n">
-        <v>46631</v>
+        <v>46539</v>
       </c>
       <c r="B55" s="21" t="n">
-        <f aca="false">IF(A55&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A55&gt;$B$40,$B$41,0)+IF(A55&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A55&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A55&gt;$B$43,$B$44,0)+IF(A55&gt;=$B$35,$B$37,0)+$B$32-IF(A55&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C55" s="12" t="n">
-        <f aca="false">IF(A55=$B$39,$B$26-$B$29,0)-IF(A55=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A55=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A55=$B$42,$B$26-$B$29,0)-IF(A55=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A55=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D55" s="12" t="n">
@@ -6195,7 +5967,7 @@
       </c>
       <c r="N55" s="12" t="n">
         <f aca="false">P54</f>
-        <v>62418.6498653134</v>
+        <v>54711.3698653134</v>
       </c>
       <c r="O55" s="12" t="n">
         <f aca="false">MIN(D55-G55-L55,MAX($B$15-$B$18-N55,0))</f>
@@ -6203,7 +5975,7 @@
       </c>
       <c r="P55" s="12" t="n">
         <f aca="false">N55+O55</f>
-        <v>64987.7431986467</v>
+        <v>57280.4631986467</v>
       </c>
       <c r="Q55" s="5" t="n">
         <f aca="false">IF(H55&lt;=0.005,1,0)</f>
@@ -6231,19 +6003,19 @@
       </c>
       <c r="W55" s="12" t="n">
         <f aca="false">P55+$B$18</f>
-        <v>81248.4931986467</v>
+        <v>73541.2131986467</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="34" t="n">
-        <v>46661</v>
+        <v>46569</v>
       </c>
       <c r="B56" s="21" t="n">
-        <f aca="false">IF(A56&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A56&gt;$B$40,$B$41,0)+IF(A56&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A56&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A56&gt;$B$43,$B$44,0)+IF(A56&gt;=$B$35,$B$37,0)+$B$32-IF(A56&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C56" s="12" t="n">
-        <f aca="false">IF(A56=$B$39,$B$26-$B$29,0)-IF(A56=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A56=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A56=$B$42,$B$26-$B$29,0)-IF(A56=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A56=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D56" s="12" t="n">
@@ -6288,7 +6060,7 @@
       </c>
       <c r="N56" s="12" t="n">
         <f aca="false">P55</f>
-        <v>64987.7431986467</v>
+        <v>57280.4631986467</v>
       </c>
       <c r="O56" s="12" t="n">
         <f aca="false">MIN(D56-G56-L56,MAX($B$15-$B$18-N56,0))</f>
@@ -6296,7 +6068,7 @@
       </c>
       <c r="P56" s="12" t="n">
         <f aca="false">N56+O56</f>
-        <v>67556.83653198</v>
+        <v>59849.55653198</v>
       </c>
       <c r="Q56" s="5" t="n">
         <f aca="false">IF(H56&lt;=0.005,1,0)</f>
@@ -6324,19 +6096,19 @@
       </c>
       <c r="W56" s="12" t="n">
         <f aca="false">P56+$B$18</f>
-        <v>83817.58653198</v>
+        <v>76110.30653198</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="34" t="n">
-        <v>46692</v>
+        <v>46600</v>
       </c>
       <c r="B57" s="21" t="n">
-        <f aca="false">IF(A57&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A57&gt;$B$40,$B$41,0)+IF(A57&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A57&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A57&gt;$B$43,$B$44,0)+IF(A57&gt;=$B$35,$B$37,0)+$B$32-IF(A57&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C57" s="12" t="n">
-        <f aca="false">IF(A57=$B$39,$B$26-$B$29,0)-IF(A57=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A57=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A57=$B$42,$B$26-$B$29,0)-IF(A57=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A57=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D57" s="12" t="n">
@@ -6381,7 +6153,7 @@
       </c>
       <c r="N57" s="12" t="n">
         <f aca="false">P56</f>
-        <v>67556.83653198</v>
+        <v>59849.55653198</v>
       </c>
       <c r="O57" s="12" t="n">
         <f aca="false">MIN(D57-G57-L57,MAX($B$15-$B$18-N57,0))</f>
@@ -6389,7 +6161,7 @@
       </c>
       <c r="P57" s="12" t="n">
         <f aca="false">N57+O57</f>
-        <v>70125.9298653134</v>
+        <v>62418.6498653134</v>
       </c>
       <c r="Q57" s="5" t="n">
         <f aca="false">IF(H57&lt;=0.005,1,0)</f>
@@ -6417,19 +6189,19 @@
       </c>
       <c r="W57" s="12" t="n">
         <f aca="false">P57+$B$18</f>
-        <v>86386.6798653134</v>
+        <v>78679.3998653134</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="34" t="n">
-        <v>46722</v>
+        <v>46631</v>
       </c>
       <c r="B58" s="21" t="n">
-        <f aca="false">IF(A58&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A58&gt;$B$40,$B$41,0)+IF(A58&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A58&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A58&gt;$B$43,$B$44,0)+IF(A58&gt;=$B$35,$B$37,0)+$B$32-IF(A58&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C58" s="12" t="n">
-        <f aca="false">IF(A58=$B$39,$B$26-$B$29,0)-IF(A58=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A58=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A58=$B$42,$B$26-$B$29,0)-IF(A58=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A58=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D58" s="12" t="n">
@@ -6474,7 +6246,7 @@
       </c>
       <c r="N58" s="12" t="n">
         <f aca="false">P57</f>
-        <v>70125.9298653134</v>
+        <v>62418.6498653134</v>
       </c>
       <c r="O58" s="12" t="n">
         <f aca="false">MIN(D58-G58-L58,MAX($B$15-$B$18-N58,0))</f>
@@ -6482,7 +6254,7 @@
       </c>
       <c r="P58" s="12" t="n">
         <f aca="false">N58+O58</f>
-        <v>72695.0231986467</v>
+        <v>64987.7431986467</v>
       </c>
       <c r="Q58" s="5" t="n">
         <f aca="false">IF(H58&lt;=0.005,1,0)</f>
@@ -6510,19 +6282,19 @@
       </c>
       <c r="W58" s="12" t="n">
         <f aca="false">P58+$B$18</f>
-        <v>88955.7731986467</v>
+        <v>81248.4931986467</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="34" t="n">
-        <v>46753</v>
+        <v>46661</v>
       </c>
       <c r="B59" s="21" t="n">
-        <f aca="false">IF(A59&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A59&gt;$B$40,$B$41,0)+IF(A59&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A59&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A59&gt;$B$43,$B$44,0)+IF(A59&gt;=$B$35,$B$37,0)+$B$32-IF(A59&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C59" s="12" t="n">
-        <f aca="false">IF(A59=$B$39,$B$26-$B$29,0)-IF(A59=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A59=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A59=$B$42,$B$26-$B$29,0)-IF(A59=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A59=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D59" s="12" t="n">
@@ -6567,7 +6339,7 @@
       </c>
       <c r="N59" s="12" t="n">
         <f aca="false">P58</f>
-        <v>72695.0231986467</v>
+        <v>64987.7431986467</v>
       </c>
       <c r="O59" s="12" t="n">
         <f aca="false">MIN(D59-G59-L59,MAX($B$15-$B$18-N59,0))</f>
@@ -6575,7 +6347,7 @@
       </c>
       <c r="P59" s="12" t="n">
         <f aca="false">N59+O59</f>
-        <v>75264.1165319801</v>
+        <v>67556.83653198</v>
       </c>
       <c r="Q59" s="5" t="n">
         <f aca="false">IF(H59&lt;=0.005,1,0)</f>
@@ -6603,19 +6375,19 @@
       </c>
       <c r="W59" s="12" t="n">
         <f aca="false">P59+$B$18</f>
-        <v>91524.8665319801</v>
+        <v>83817.58653198</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="34" t="n">
-        <v>46784</v>
+        <v>46692</v>
       </c>
       <c r="B60" s="21" t="n">
-        <f aca="false">IF(A60&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A60&gt;$B$40,$B$41,0)+IF(A60&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A60&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A60&gt;$B$43,$B$44,0)+IF(A60&gt;=$B$35,$B$37,0)+$B$32-IF(A60&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C60" s="12" t="n">
-        <f aca="false">IF(A60=$B$39,$B$26-$B$29,0)-IF(A60=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A60=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A60=$B$42,$B$26-$B$29,0)-IF(A60=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A60=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D60" s="12" t="n">
@@ -6660,7 +6432,7 @@
       </c>
       <c r="N60" s="12" t="n">
         <f aca="false">P59</f>
-        <v>75264.1165319801</v>
+        <v>67556.83653198</v>
       </c>
       <c r="O60" s="12" t="n">
         <f aca="false">MIN(D60-G60-L60,MAX($B$15-$B$18-N60,0))</f>
@@ -6668,7 +6440,7 @@
       </c>
       <c r="P60" s="12" t="n">
         <f aca="false">N60+O60</f>
-        <v>77833.2098653134</v>
+        <v>70125.9298653134</v>
       </c>
       <c r="Q60" s="5" t="n">
         <f aca="false">IF(H60&lt;=0.005,1,0)</f>
@@ -6696,19 +6468,19 @@
       </c>
       <c r="W60" s="12" t="n">
         <f aca="false">P60+$B$18</f>
-        <v>94093.9598653134</v>
+        <v>86386.6798653134</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="34" t="n">
-        <v>46813</v>
+        <v>46722</v>
       </c>
       <c r="B61" s="21" t="n">
-        <f aca="false">IF(A61&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A61&gt;$B$40,$B$41,0)+IF(A61&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A61&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A61&gt;$B$43,$B$44,0)+IF(A61&gt;=$B$35,$B$37,0)+$B$32-IF(A61&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C61" s="12" t="n">
-        <f aca="false">IF(A61=$B$39,$B$26-$B$29,0)-IF(A61=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A61=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A61=$B$42,$B$26-$B$29,0)-IF(A61=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A61=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D61" s="12" t="n">
@@ -6753,7 +6525,7 @@
       </c>
       <c r="N61" s="12" t="n">
         <f aca="false">P60</f>
-        <v>77833.2098653134</v>
+        <v>70125.9298653134</v>
       </c>
       <c r="O61" s="12" t="n">
         <f aca="false">MIN(D61-G61-L61,MAX($B$15-$B$18-N61,0))</f>
@@ -6761,7 +6533,7 @@
       </c>
       <c r="P61" s="12" t="n">
         <f aca="false">N61+O61</f>
-        <v>80402.3031986467</v>
+        <v>72695.0231986467</v>
       </c>
       <c r="Q61" s="5" t="n">
         <f aca="false">IF(H61&lt;=0.005,1,0)</f>
@@ -6789,19 +6561,19 @@
       </c>
       <c r="W61" s="12" t="n">
         <f aca="false">P61+$B$18</f>
-        <v>96663.0531986467</v>
+        <v>88955.7731986467</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="34" t="n">
-        <v>46844</v>
+        <v>46753</v>
       </c>
       <c r="B62" s="21" t="n">
-        <f aca="false">IF(A62&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A62&gt;$B$40,$B$41,0)+IF(A62&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A62&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A62&gt;$B$43,$B$44,0)+IF(A62&gt;=$B$35,$B$37,0)+$B$32-IF(A62&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C62" s="12" t="n">
-        <f aca="false">IF(A62=$B$39,$B$26-$B$29,0)-IF(A62=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A62=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A62=$B$42,$B$26-$B$29,0)-IF(A62=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A62=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D62" s="12" t="n">
@@ -6846,7 +6618,7 @@
       </c>
       <c r="N62" s="12" t="n">
         <f aca="false">P61</f>
-        <v>80402.3031986467</v>
+        <v>72695.0231986467</v>
       </c>
       <c r="O62" s="12" t="n">
         <f aca="false">MIN(D62-G62-L62,MAX($B$15-$B$18-N62,0))</f>
@@ -6854,7 +6626,7 @@
       </c>
       <c r="P62" s="12" t="n">
         <f aca="false">N62+O62</f>
-        <v>82971.3965319801</v>
+        <v>75264.1165319801</v>
       </c>
       <c r="Q62" s="5" t="n">
         <f aca="false">IF(H62&lt;=0.005,1,0)</f>
@@ -6882,19 +6654,19 @@
       </c>
       <c r="W62" s="12" t="n">
         <f aca="false">P62+$B$18</f>
-        <v>99232.1465319801</v>
+        <v>91524.8665319801</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="34" t="n">
-        <v>46874</v>
+        <v>46784</v>
       </c>
       <c r="B63" s="21" t="n">
-        <f aca="false">IF(A63&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A63&gt;$B$40,$B$41,0)+IF(A63&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A63&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A63&gt;$B$43,$B$44,0)+IF(A63&gt;=$B$35,$B$37,0)+$B$32-IF(A63&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C63" s="12" t="n">
-        <f aca="false">IF(A63=$B$39,$B$26-$B$29,0)-IF(A63=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A63=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A63=$B$42,$B$26-$B$29,0)-IF(A63=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A63=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D63" s="12" t="n">
@@ -6939,15 +6711,15 @@
       </c>
       <c r="N63" s="12" t="n">
         <f aca="false">P62</f>
-        <v>82971.3965319801</v>
+        <v>75264.1165319801</v>
       </c>
       <c r="O63" s="12" t="n">
         <f aca="false">MIN(D63-G63-L63,MAX($B$15-$B$18-N63,0))</f>
-        <v>1609.85346801994</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="P63" s="12" t="n">
         <f aca="false">N63+O63</f>
-        <v>84581.25</v>
+        <v>77833.2098653134</v>
       </c>
       <c r="Q63" s="5" t="n">
         <f aca="false">IF(H63&lt;=0.005,1,0)</f>
@@ -6967,27 +6739,27 @@
       </c>
       <c r="U63" s="5" t="n">
         <f aca="false">IF(P63+$B$18&gt;=$B$15-0.5,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V63" s="12" t="n">
         <f aca="false">MAX(D63-G63-L63,0)-MAX(O63,0)</f>
-        <v>959.239865313398</v>
+        <v>0</v>
       </c>
       <c r="W63" s="12" t="n">
         <f aca="false">P63+$B$18</f>
-        <v>100842</v>
+        <v>94093.9598653134</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="34" t="n">
-        <v>46905</v>
+        <v>46813</v>
       </c>
       <c r="B64" s="21" t="n">
-        <f aca="false">IF(A64&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A64&gt;$B$40,$B$41,0)+IF(A64&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A64&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A64&gt;$B$43,$B$44,0)+IF(A64&gt;=$B$35,$B$37,0)+$B$32-IF(A64&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C64" s="12" t="n">
-        <f aca="false">IF(A64=$B$39,$B$26-$B$29,0)-IF(A64=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A64=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A64=$B$42,$B$26-$B$29,0)-IF(A64=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A64=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D64" s="12" t="n">
@@ -7032,15 +6804,15 @@
       </c>
       <c r="N64" s="12" t="n">
         <f aca="false">P63</f>
-        <v>84581.25</v>
+        <v>77833.2098653134</v>
       </c>
       <c r="O64" s="12" t="n">
         <f aca="false">MIN(D64-G64-L64,MAX($B$15-$B$18-N64,0))</f>
-        <v>0</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="P64" s="12" t="n">
         <f aca="false">N64+O64</f>
-        <v>84581.25</v>
+        <v>80402.3031986467</v>
       </c>
       <c r="Q64" s="5" t="n">
         <f aca="false">IF(H64&lt;=0.005,1,0)</f>
@@ -7060,27 +6832,27 @@
       </c>
       <c r="U64" s="5" t="n">
         <f aca="false">IF(P64+$B$18&gt;=$B$15-0.5,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V64" s="12" t="n">
         <f aca="false">MAX(D64-G64-L64,0)-MAX(O64,0)</f>
-        <v>2569.09333333334</v>
+        <v>0</v>
       </c>
       <c r="W64" s="12" t="n">
         <f aca="false">P64+$B$18</f>
-        <v>100842</v>
+        <v>96663.0531986467</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="34" t="n">
-        <v>46935</v>
+        <v>46844</v>
       </c>
       <c r="B65" s="21" t="n">
-        <f aca="false">IF(A65&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A65&gt;$B$40,$B$41,0)+IF(A65&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A65&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A65&gt;$B$43,$B$44,0)+IF(A65&gt;=$B$35,$B$37,0)+$B$32-IF(A65&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C65" s="12" t="n">
-        <f aca="false">IF(A65=$B$39,$B$26-$B$29,0)-IF(A65=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A65=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A65=$B$42,$B$26-$B$29,0)-IF(A65=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A65=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D65" s="12" t="n">
@@ -7125,15 +6897,15 @@
       </c>
       <c r="N65" s="12" t="n">
         <f aca="false">P64</f>
-        <v>84581.25</v>
+        <v>80402.3031986467</v>
       </c>
       <c r="O65" s="12" t="n">
         <f aca="false">MIN(D65-G65-L65,MAX($B$15-$B$18-N65,0))</f>
-        <v>0</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="P65" s="12" t="n">
         <f aca="false">N65+O65</f>
-        <v>84581.25</v>
+        <v>82971.3965319801</v>
       </c>
       <c r="Q65" s="5" t="n">
         <f aca="false">IF(H65&lt;=0.005,1,0)</f>
@@ -7153,27 +6925,27 @@
       </c>
       <c r="U65" s="5" t="n">
         <f aca="false">IF(P65+$B$18&gt;=$B$15-0.5,1,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V65" s="12" t="n">
         <f aca="false">MAX(D65-G65-L65,0)-MAX(O65,0)</f>
-        <v>2569.09333333334</v>
+        <v>0</v>
       </c>
       <c r="W65" s="12" t="n">
         <f aca="false">P65+$B$18</f>
-        <v>100842</v>
+        <v>99232.1465319801</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="34" t="n">
-        <v>46966</v>
+        <v>46874</v>
       </c>
       <c r="B66" s="21" t="n">
-        <f aca="false">IF(A66&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A66&gt;$B$40,$B$41,0)+IF(A66&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A66&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A66&gt;$B$43,$B$44,0)+IF(A66&gt;=$B$35,$B$37,0)+$B$32-IF(A66&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C66" s="12" t="n">
-        <f aca="false">IF(A66=$B$39,$B$26-$B$29,0)-IF(A66=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A66=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A66=$B$42,$B$26-$B$29,0)-IF(A66=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A66=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D66" s="12" t="n">
@@ -7218,11 +6990,11 @@
       </c>
       <c r="N66" s="12" t="n">
         <f aca="false">P65</f>
-        <v>84581.25</v>
+        <v>82971.3965319801</v>
       </c>
       <c r="O66" s="12" t="n">
         <f aca="false">MIN(D66-G66-L66,MAX($B$15-$B$18-N66,0))</f>
-        <v>0</v>
+        <v>1609.85346801994</v>
       </c>
       <c r="P66" s="12" t="n">
         <f aca="false">N66+O66</f>
@@ -7250,7 +7022,7 @@
       </c>
       <c r="V66" s="12" t="n">
         <f aca="false">MAX(D66-G66-L66,0)-MAX(O66,0)</f>
-        <v>2569.09333333334</v>
+        <v>959.239865313398</v>
       </c>
       <c r="W66" s="12" t="n">
         <f aca="false">P66+$B$18</f>
@@ -7259,14 +7031,14 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="34" t="n">
-        <v>46997</v>
+        <v>46905</v>
       </c>
       <c r="B67" s="21" t="n">
-        <f aca="false">IF(A67&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A67&gt;$B$40,$B$41,0)+IF(A67&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A67&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A67&gt;$B$43,$B$44,0)+IF(A67&gt;=$B$35,$B$37,0)+$B$32-IF(A67&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C67" s="12" t="n">
-        <f aca="false">IF(A67=$B$39,$B$26-$B$29,0)-IF(A67=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A67=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A67=$B$42,$B$26-$B$29,0)-IF(A67=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A67=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D67" s="12" t="n">
@@ -7352,14 +7124,14 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="34" t="n">
-        <v>47027</v>
+        <v>46935</v>
       </c>
       <c r="B68" s="21" t="n">
-        <f aca="false">IF(A68&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A68&gt;$B$40,$B$41,0)+IF(A68&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A68&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A68&gt;$B$43,$B$44,0)+IF(A68&gt;=$B$35,$B$37,0)+$B$32-IF(A68&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C68" s="12" t="n">
-        <f aca="false">IF(A68=$B$39,$B$26-$B$29,0)-IF(A68=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A68=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A68=$B$42,$B$26-$B$29,0)-IF(A68=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A68=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D68" s="12" t="n">
@@ -7445,14 +7217,14 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="34" t="n">
-        <v>47058</v>
+        <v>46966</v>
       </c>
       <c r="B69" s="21" t="n">
-        <f aca="false">IF(A69&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A69&gt;$B$40,$B$41,0)+IF(A69&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A69&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A69&gt;$B$43,$B$44,0)+IF(A69&gt;=$B$35,$B$37,0)+$B$32-IF(A69&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C69" s="12" t="n">
-        <f aca="false">IF(A69=$B$39,$B$26-$B$29,0)-IF(A69=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A69=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A69=$B$42,$B$26-$B$29,0)-IF(A69=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A69=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D69" s="12" t="n">
@@ -7538,14 +7310,14 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="34" t="n">
-        <v>47088</v>
+        <v>46997</v>
       </c>
       <c r="B70" s="21" t="n">
-        <f aca="false">IF(A70&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A70&gt;$B$40,$B$41,0)+IF(A70&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A70&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A70&gt;$B$43,$B$44,0)+IF(A70&gt;=$B$35,$B$37,0)+$B$32-IF(A70&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C70" s="12" t="n">
-        <f aca="false">IF(A70=$B$39,$B$26-$B$29,0)-IF(A70=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A70=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A70=$B$42,$B$26-$B$29,0)-IF(A70=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A70=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D70" s="12" t="n">
@@ -7631,14 +7403,14 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="34" t="n">
-        <v>47119</v>
+        <v>47027</v>
       </c>
       <c r="B71" s="21" t="n">
-        <f aca="false">IF(A71&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A71&gt;$B$40,$B$41,0)+IF(A71&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A71&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A71&gt;$B$43,$B$44,0)+IF(A71&gt;=$B$35,$B$37,0)+$B$32-IF(A71&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2569.09333333334</v>
       </c>
       <c r="C71" s="12" t="n">
-        <f aca="false">IF(A71=$B$39,$B$26-$B$29,0)-IF(A71=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A71=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A71=$B$42,$B$26-$B$29,0)-IF(A71=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A71=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D71" s="12" t="n">
@@ -7724,19 +7496,19 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="34" t="n">
-        <v>47150</v>
+        <v>47058</v>
       </c>
       <c r="B72" s="21" t="n">
-        <f aca="false">IF(A72&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A72&gt;$B$40,$B$41,0)+IF(A72&gt;=$B$35,$B$37,0)+$B$32</f>
-        <v>2911.09333333334</v>
+        <f aca="false">IF(A72&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A72&gt;$B$43,$B$44,0)+IF(A72&gt;=$B$35,$B$37,0)+$B$32-IF(A72&gt;=$B$40,$B$39*(1-$B$41),0)</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C72" s="12" t="n">
-        <f aca="false">IF(A72=$B$39,$B$26-$B$29,0)-IF(A72=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A72=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A72=$B$42,$B$26-$B$29,0)-IF(A72=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A72=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D72" s="12" t="n">
         <f aca="false">B72+C72</f>
-        <v>2911.09333333334</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E72" s="12" t="n">
         <f aca="false">H71</f>
@@ -7808,7 +7580,7 @@
       </c>
       <c r="V72" s="12" t="n">
         <f aca="false">MAX(D72-G72-L72,0)-MAX(O72,0)</f>
-        <v>2911.09333333334</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="W72" s="12" t="n">
         <f aca="false">P72+$B$18</f>
@@ -7817,19 +7589,19 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="34" t="n">
-        <v>47178</v>
+        <v>47088</v>
       </c>
       <c r="B73" s="21" t="n">
-        <f aca="false">IF(A73&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A73&gt;$B$40,$B$41,0)+IF(A73&gt;=$B$35,$B$37,0)+$B$32</f>
-        <v>2911.09333333334</v>
+        <f aca="false">IF(A73&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A73&gt;$B$43,$B$44,0)+IF(A73&gt;=$B$35,$B$37,0)+$B$32-IF(A73&gt;=$B$40,$B$39*(1-$B$41),0)</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C73" s="12" t="n">
-        <f aca="false">IF(A73=$B$39,$B$26-$B$29,0)-IF(A73=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A73=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A73=$B$42,$B$26-$B$29,0)-IF(A73=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A73=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D73" s="12" t="n">
         <f aca="false">B73+C73</f>
-        <v>2911.09333333334</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E73" s="12" t="n">
         <f aca="false">H72</f>
@@ -7901,7 +7673,7 @@
       </c>
       <c r="V73" s="12" t="n">
         <f aca="false">MAX(D73-G73-L73,0)-MAX(O73,0)</f>
-        <v>2911.09333333334</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="W73" s="12" t="n">
         <f aca="false">P73+$B$18</f>
@@ -7910,19 +7682,19 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="34" t="n">
-        <v>47209</v>
+        <v>47119</v>
       </c>
       <c r="B74" s="21" t="n">
-        <f aca="false">IF(A74&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A74&gt;$B$40,$B$41,0)+IF(A74&gt;=$B$35,$B$37,0)+$B$32</f>
-        <v>2911.09333333334</v>
+        <f aca="false">IF(A74&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A74&gt;$B$43,$B$44,0)+IF(A74&gt;=$B$35,$B$37,0)+$B$32-IF(A74&gt;=$B$40,$B$39*(1-$B$41),0)</f>
+        <v>2569.09333333334</v>
       </c>
       <c r="C74" s="12" t="n">
-        <f aca="false">IF(A74=$B$39,$B$26-$B$29,0)-IF(A74=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A74=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A74=$B$42,$B$26-$B$29,0)-IF(A74=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A74=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D74" s="12" t="n">
         <f aca="false">B74+C74</f>
-        <v>2911.09333333334</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="E74" s="12" t="n">
         <f aca="false">H73</f>
@@ -7994,7 +7766,7 @@
       </c>
       <c r="V74" s="12" t="n">
         <f aca="false">MAX(D74-G74-L74,0)-MAX(O74,0)</f>
-        <v>2911.09333333334</v>
+        <v>2569.09333333334</v>
       </c>
       <c r="W74" s="12" t="n">
         <f aca="false">P74+$B$18</f>
@@ -8003,14 +7775,14 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="34" t="n">
-        <v>47239</v>
+        <v>47150</v>
       </c>
       <c r="B75" s="21" t="n">
-        <f aca="false">IF(A75&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A75&gt;$B$40,$B$41,0)+IF(A75&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A75&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A75&gt;$B$43,$B$44,0)+IF(A75&gt;=$B$35,$B$37,0)+$B$32-IF(A75&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C75" s="12" t="n">
-        <f aca="false">IF(A75=$B$39,$B$26-$B$29,0)-IF(A75=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A75=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A75=$B$42,$B$26-$B$29,0)-IF(A75=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A75=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D75" s="12" t="n">
@@ -8096,14 +7868,14 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="34" t="n">
-        <v>47270</v>
+        <v>47178</v>
       </c>
       <c r="B76" s="21" t="n">
-        <f aca="false">IF(A76&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A76&gt;$B$40,$B$41,0)+IF(A76&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A76&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A76&gt;$B$43,$B$44,0)+IF(A76&gt;=$B$35,$B$37,0)+$B$32-IF(A76&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C76" s="12" t="n">
-        <f aca="false">IF(A76=$B$39,$B$26-$B$29,0)-IF(A76=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A76=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A76=$B$42,$B$26-$B$29,0)-IF(A76=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A76=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D76" s="12" t="n">
@@ -8189,14 +7961,14 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="34" t="n">
-        <v>47300</v>
+        <v>47209</v>
       </c>
       <c r="B77" s="21" t="n">
-        <f aca="false">IF(A77&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A77&gt;$B$40,$B$41,0)+IF(A77&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A77&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A77&gt;$B$43,$B$44,0)+IF(A77&gt;=$B$35,$B$37,0)+$B$32-IF(A77&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C77" s="12" t="n">
-        <f aca="false">IF(A77=$B$39,$B$26-$B$29,0)-IF(A77=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A77=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A77=$B$42,$B$26-$B$29,0)-IF(A77=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A77=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D77" s="12" t="n">
@@ -8282,14 +8054,14 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="34" t="n">
-        <v>47331</v>
+        <v>47239</v>
       </c>
       <c r="B78" s="21" t="n">
-        <f aca="false">IF(A78&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A78&gt;$B$40,$B$41,0)+IF(A78&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A78&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A78&gt;$B$43,$B$44,0)+IF(A78&gt;=$B$35,$B$37,0)+$B$32-IF(A78&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C78" s="12" t="n">
-        <f aca="false">IF(A78=$B$39,$B$26-$B$29,0)-IF(A78=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A78=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A78=$B$42,$B$26-$B$29,0)-IF(A78=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A78=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D78" s="12" t="n">
@@ -8375,14 +8147,14 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="34" t="n">
-        <v>47362</v>
+        <v>47270</v>
       </c>
       <c r="B79" s="21" t="n">
-        <f aca="false">IF(A79&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A79&gt;$B$40,$B$41,0)+IF(A79&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A79&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A79&gt;$B$43,$B$44,0)+IF(A79&gt;=$B$35,$B$37,0)+$B$32-IF(A79&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C79" s="12" t="n">
-        <f aca="false">IF(A79=$B$39,$B$26-$B$29,0)-IF(A79=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A79=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A79=$B$42,$B$26-$B$29,0)-IF(A79=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A79=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D79" s="12" t="n">
@@ -8468,14 +8240,14 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="34" t="n">
-        <v>47392</v>
+        <v>47300</v>
       </c>
       <c r="B80" s="21" t="n">
-        <f aca="false">IF(A80&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A80&gt;$B$40,$B$41,0)+IF(A80&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A80&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A80&gt;$B$43,$B$44,0)+IF(A80&gt;=$B$35,$B$37,0)+$B$32-IF(A80&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C80" s="12" t="n">
-        <f aca="false">IF(A80=$B$39,$B$26-$B$29,0)-IF(A80=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A80=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A80=$B$42,$B$26-$B$29,0)-IF(A80=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A80=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D80" s="12" t="n">
@@ -8561,14 +8333,14 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="34" t="n">
-        <v>47423</v>
+        <v>47331</v>
       </c>
       <c r="B81" s="21" t="n">
-        <f aca="false">IF(A81&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A81&gt;$B$40,$B$41,0)+IF(A81&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A81&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A81&gt;$B$43,$B$44,0)+IF(A81&gt;=$B$35,$B$37,0)+$B$32-IF(A81&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C81" s="12" t="n">
-        <f aca="false">IF(A81=$B$39,$B$26-$B$29,0)-IF(A81=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A81=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A81=$B$42,$B$26-$B$29,0)-IF(A81=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A81=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D81" s="12" t="n">
@@ -8654,14 +8426,14 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="34" t="n">
-        <v>47453</v>
+        <v>47362</v>
       </c>
       <c r="B82" s="21" t="n">
-        <f aca="false">IF(A82&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A82&gt;$B$40,$B$41,0)+IF(A82&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A82&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A82&gt;$B$43,$B$44,0)+IF(A82&gt;=$B$35,$B$37,0)+$B$32-IF(A82&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C82" s="12" t="n">
-        <f aca="false">IF(A82=$B$39,$B$26-$B$29,0)-IF(A82=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A82=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A82=$B$42,$B$26-$B$29,0)-IF(A82=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A82=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D82" s="12" t="n">
@@ -8747,14 +8519,14 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="34" t="n">
-        <v>47484</v>
+        <v>47392</v>
       </c>
       <c r="B83" s="21" t="n">
-        <f aca="false">IF(A83&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A83&gt;$B$40,$B$41,0)+IF(A83&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A83&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A83&gt;$B$43,$B$44,0)+IF(A83&gt;=$B$35,$B$37,0)+$B$32-IF(A83&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C83" s="12" t="n">
-        <f aca="false">IF(A83=$B$39,$B$26-$B$29,0)-IF(A83=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A83=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A83=$B$42,$B$26-$B$29,0)-IF(A83=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A83=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D83" s="12" t="n">
@@ -8840,14 +8612,14 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="34" t="n">
-        <v>47515</v>
+        <v>47423</v>
       </c>
       <c r="B84" s="21" t="n">
-        <f aca="false">IF(A84&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A84&gt;$B$40,$B$41,0)+IF(A84&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A84&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A84&gt;$B$43,$B$44,0)+IF(A84&gt;=$B$35,$B$37,0)+$B$32-IF(A84&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C84" s="12" t="n">
-        <f aca="false">IF(A84=$B$39,$B$26-$B$29,0)-IF(A84=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A84=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A84=$B$42,$B$26-$B$29,0)-IF(A84=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A84=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D84" s="12" t="n">
@@ -8933,14 +8705,14 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="34" t="n">
-        <v>47543</v>
+        <v>47453</v>
       </c>
       <c r="B85" s="21" t="n">
-        <f aca="false">IF(A85&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A85&gt;$B$40,$B$41,0)+IF(A85&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A85&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A85&gt;$B$43,$B$44,0)+IF(A85&gt;=$B$35,$B$37,0)+$B$32-IF(A85&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C85" s="12" t="n">
-        <f aca="false">IF(A85=$B$39,$B$26-$B$29,0)-IF(A85=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A85=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A85=$B$42,$B$26-$B$29,0)-IF(A85=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A85=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D85" s="12" t="n">
@@ -9026,14 +8798,14 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="34" t="n">
-        <v>47574</v>
+        <v>47484</v>
       </c>
       <c r="B86" s="21" t="n">
-        <f aca="false">IF(A86&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A86&gt;$B$40,$B$41,0)+IF(A86&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A86&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A86&gt;$B$43,$B$44,0)+IF(A86&gt;=$B$35,$B$37,0)+$B$32-IF(A86&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C86" s="12" t="n">
-        <f aca="false">IF(A86=$B$39,$B$26-$B$29,0)-IF(A86=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A86=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A86=$B$42,$B$26-$B$29,0)-IF(A86=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A86=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D86" s="12" t="n">
@@ -9119,14 +8891,14 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="34" t="n">
-        <v>47604</v>
+        <v>47515</v>
       </c>
       <c r="B87" s="21" t="n">
-        <f aca="false">IF(A87&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A87&gt;$B$40,$B$41,0)+IF(A87&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A87&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A87&gt;$B$43,$B$44,0)+IF(A87&gt;=$B$35,$B$37,0)+$B$32-IF(A87&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C87" s="12" t="n">
-        <f aca="false">IF(A87=$B$39,$B$26-$B$29,0)-IF(A87=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A87=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A87=$B$42,$B$26-$B$29,0)-IF(A87=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A87=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D87" s="12" t="n">
@@ -9212,14 +8984,14 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="34" t="n">
-        <v>47635</v>
+        <v>47543</v>
       </c>
       <c r="B88" s="21" t="n">
-        <f aca="false">IF(A88&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A88&gt;$B$40,$B$41,0)+IF(A88&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A88&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A88&gt;$B$43,$B$44,0)+IF(A88&gt;=$B$35,$B$37,0)+$B$32-IF(A88&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C88" s="12" t="n">
-        <f aca="false">IF(A88=$B$39,$B$26-$B$29,0)-IF(A88=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A88=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A88=$B$42,$B$26-$B$29,0)-IF(A88=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A88=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D88" s="12" t="n">
@@ -9305,14 +9077,14 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="34" t="n">
-        <v>47665</v>
+        <v>47574</v>
       </c>
       <c r="B89" s="21" t="n">
-        <f aca="false">IF(A89&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A89&gt;$B$40,$B$41,0)+IF(A89&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A89&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A89&gt;$B$43,$B$44,0)+IF(A89&gt;=$B$35,$B$37,0)+$B$32-IF(A89&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C89" s="12" t="n">
-        <f aca="false">IF(A89=$B$39,$B$26-$B$29,0)-IF(A89=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A89=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A89=$B$42,$B$26-$B$29,0)-IF(A89=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A89=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D89" s="12" t="n">
@@ -9398,14 +9170,14 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="34" t="n">
-        <v>47696</v>
+        <v>47604</v>
       </c>
       <c r="B90" s="21" t="n">
-        <f aca="false">IF(A90&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A90&gt;$B$40,$B$41,0)+IF(A90&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A90&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A90&gt;$B$43,$B$44,0)+IF(A90&gt;=$B$35,$B$37,0)+$B$32-IF(A90&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C90" s="12" t="n">
-        <f aca="false">IF(A90=$B$39,$B$26-$B$29,0)-IF(A90=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A90=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A90=$B$42,$B$26-$B$29,0)-IF(A90=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A90=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D90" s="12" t="n">
@@ -9491,14 +9263,14 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="34" t="n">
-        <v>47727</v>
+        <v>47635</v>
       </c>
       <c r="B91" s="21" t="n">
-        <f aca="false">IF(A91&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A91&gt;$B$40,$B$41,0)+IF(A91&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A91&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A91&gt;$B$43,$B$44,0)+IF(A91&gt;=$B$35,$B$37,0)+$B$32-IF(A91&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C91" s="12" t="n">
-        <f aca="false">IF(A91=$B$39,$B$26-$B$29,0)-IF(A91=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A91=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A91=$B$42,$B$26-$B$29,0)-IF(A91=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A91=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D91" s="12" t="n">
@@ -9584,14 +9356,14 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="34" t="n">
-        <v>47757</v>
+        <v>47665</v>
       </c>
       <c r="B92" s="21" t="n">
-        <f aca="false">IF(A92&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A92&gt;$B$40,$B$41,0)+IF(A92&gt;=$B$35,$B$37,0)+$B$32</f>
+        <f aca="false">IF(A92&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A92&gt;$B$43,$B$44,0)+IF(A92&gt;=$B$35,$B$37,0)+$B$32-IF(A92&gt;=$B$40,$B$39*(1-$B$41),0)</f>
         <v>2911.09333333334</v>
       </c>
       <c r="C92" s="12" t="n">
-        <f aca="false">IF(A92=$B$39,$B$26-$B$29,0)-IF(A92=DATE(YEAR($B$39),MONTH($B$39)+1,1),$B$28,0)+IF(A92=$B$35,$B$37*$B$36,0)+0</f>
+        <f aca="false">IF(A92=$B$42,$B$26-$B$29,0)-IF(A92=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A92=$B$35,$B$37*$B$36,0)+0</f>
         <v>0</v>
       </c>
       <c r="D92" s="12" t="n">
@@ -9672,6 +9444,285 @@
       </c>
       <c r="W92" s="12" t="n">
         <f aca="false">P92+$B$18</f>
+        <v>100842</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="34" t="n">
+        <v>47696</v>
+      </c>
+      <c r="B93" s="21" t="n">
+        <f aca="false">IF(A93&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A93&gt;$B$43,$B$44,0)+IF(A93&gt;=$B$35,$B$37,0)+$B$32-IF(A93&gt;=$B$40,$B$39*(1-$B$41),0)</f>
+        <v>2911.09333333334</v>
+      </c>
+      <c r="C93" s="12" t="n">
+        <f aca="false">IF(A93=$B$42,$B$26-$B$29,0)-IF(A93=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A93=$B$35,$B$37*$B$36,0)+0</f>
+        <v>0</v>
+      </c>
+      <c r="D93" s="12" t="n">
+        <f aca="false">B93+C93</f>
+        <v>2911.09333333334</v>
+      </c>
+      <c r="E93" s="12" t="n">
+        <f aca="false">H92</f>
+        <v>0</v>
+      </c>
+      <c r="F93" s="12" t="n">
+        <f aca="false">E93*$B$6/12</f>
+        <v>0</v>
+      </c>
+      <c r="G93" s="12" t="n">
+        <f aca="false">MIN(E93+F93,MAX(D93-K93,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H93" s="12" t="n">
+        <f aca="false">E93+F93-G93</f>
+        <v>0</v>
+      </c>
+      <c r="I93" s="12" t="n">
+        <f aca="false">M92</f>
+        <v>0</v>
+      </c>
+      <c r="J93" s="12" t="n">
+        <f aca="false">I93*$B$8/12</f>
+        <v>0</v>
+      </c>
+      <c r="K93" s="12" t="n">
+        <f aca="false">MIN(I93+J93,J93+$B$9*I93)</f>
+        <v>0</v>
+      </c>
+      <c r="L93" s="12" t="n">
+        <f aca="false">MIN(I93+J93,MAX(D93-G93,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M93" s="12" t="n">
+        <f aca="false">I93+J93-L93</f>
+        <v>0</v>
+      </c>
+      <c r="N93" s="12" t="n">
+        <f aca="false">P92</f>
+        <v>84581.25</v>
+      </c>
+      <c r="O93" s="12" t="n">
+        <f aca="false">MIN(D93-G93-L93,MAX($B$15-$B$18-N93,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P93" s="12" t="n">
+        <f aca="false">N93+O93</f>
+        <v>84581.25</v>
+      </c>
+      <c r="Q93" s="5" t="n">
+        <f aca="false">IF(H93&lt;=0.005,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="R93" s="5" t="n">
+        <f aca="false">IF(M93&lt;=0.005,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="S93" s="5" t="n">
+        <f aca="false">IF(AND(Q93=1,R93=1),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="T93" s="5" t="n">
+        <f aca="false">IF(P93&gt;=$B$20,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="U93" s="5" t="n">
+        <f aca="false">IF(P93+$B$18&gt;=$B$15-0.5,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="V93" s="12" t="n">
+        <f aca="false">MAX(D93-G93-L93,0)-MAX(O93,0)</f>
+        <v>2911.09333333334</v>
+      </c>
+      <c r="W93" s="12" t="n">
+        <f aca="false">P93+$B$18</f>
+        <v>100842</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="34" t="n">
+        <v>47727</v>
+      </c>
+      <c r="B94" s="21" t="n">
+        <f aca="false">IF(A94&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A94&gt;$B$43,$B$44,0)+IF(A94&gt;=$B$35,$B$37,0)+$B$32-IF(A94&gt;=$B$40,$B$39*(1-$B$41),0)</f>
+        <v>2911.09333333334</v>
+      </c>
+      <c r="C94" s="12" t="n">
+        <f aca="false">IF(A94=$B$42,$B$26-$B$29,0)-IF(A94=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A94=$B$35,$B$37*$B$36,0)+0</f>
+        <v>0</v>
+      </c>
+      <c r="D94" s="12" t="n">
+        <f aca="false">B94+C94</f>
+        <v>2911.09333333334</v>
+      </c>
+      <c r="E94" s="12" t="n">
+        <f aca="false">H93</f>
+        <v>0</v>
+      </c>
+      <c r="F94" s="12" t="n">
+        <f aca="false">E94*$B$6/12</f>
+        <v>0</v>
+      </c>
+      <c r="G94" s="12" t="n">
+        <f aca="false">MIN(E94+F94,MAX(D94-K94,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H94" s="12" t="n">
+        <f aca="false">E94+F94-G94</f>
+        <v>0</v>
+      </c>
+      <c r="I94" s="12" t="n">
+        <f aca="false">M93</f>
+        <v>0</v>
+      </c>
+      <c r="J94" s="12" t="n">
+        <f aca="false">I94*$B$8/12</f>
+        <v>0</v>
+      </c>
+      <c r="K94" s="12" t="n">
+        <f aca="false">MIN(I94+J94,J94+$B$9*I94)</f>
+        <v>0</v>
+      </c>
+      <c r="L94" s="12" t="n">
+        <f aca="false">MIN(I94+J94,MAX(D94-G94,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M94" s="12" t="n">
+        <f aca="false">I94+J94-L94</f>
+        <v>0</v>
+      </c>
+      <c r="N94" s="12" t="n">
+        <f aca="false">P93</f>
+        <v>84581.25</v>
+      </c>
+      <c r="O94" s="12" t="n">
+        <f aca="false">MIN(D94-G94-L94,MAX($B$15-$B$18-N94,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P94" s="12" t="n">
+        <f aca="false">N94+O94</f>
+        <v>84581.25</v>
+      </c>
+      <c r="Q94" s="5" t="n">
+        <f aca="false">IF(H94&lt;=0.005,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="R94" s="5" t="n">
+        <f aca="false">IF(M94&lt;=0.005,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="S94" s="5" t="n">
+        <f aca="false">IF(AND(Q94=1,R94=1),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="T94" s="5" t="n">
+        <f aca="false">IF(P94&gt;=$B$20,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="U94" s="5" t="n">
+        <f aca="false">IF(P94+$B$18&gt;=$B$15-0.5,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="V94" s="12" t="n">
+        <f aca="false">MAX(D94-G94-L94,0)-MAX(O94,0)</f>
+        <v>2911.09333333334</v>
+      </c>
+      <c r="W94" s="12" t="n">
+        <f aca="false">P94+$B$18</f>
+        <v>100842</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="34" t="n">
+        <v>47757</v>
+      </c>
+      <c r="B95" s="21" t="n">
+        <f aca="false">IF(A95&lt;=$B$21,Budget!$F$70,Budget!$F$71)+IF(A95&gt;$B$43,$B$44,0)+IF(A95&gt;=$B$35,$B$37,0)+$B$32-IF(A95&gt;=$B$40,$B$39*(1-$B$41),0)</f>
+        <v>2911.09333333334</v>
+      </c>
+      <c r="C95" s="12" t="n">
+        <f aca="false">IF(A95=$B$42,$B$26-$B$29,0)-IF(A95=DATE(YEAR($B$42),MONTH($B$42)+1,1),$B$28,0)+IF(A95=$B$35,$B$37*$B$36,0)+0</f>
+        <v>0</v>
+      </c>
+      <c r="D95" s="12" t="n">
+        <f aca="false">B95+C95</f>
+        <v>2911.09333333334</v>
+      </c>
+      <c r="E95" s="12" t="n">
+        <f aca="false">H94</f>
+        <v>0</v>
+      </c>
+      <c r="F95" s="12" t="n">
+        <f aca="false">E95*$B$6/12</f>
+        <v>0</v>
+      </c>
+      <c r="G95" s="12" t="n">
+        <f aca="false">MIN(E95+F95,MAX(D95-K95,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H95" s="12" t="n">
+        <f aca="false">E95+F95-G95</f>
+        <v>0</v>
+      </c>
+      <c r="I95" s="12" t="n">
+        <f aca="false">M94</f>
+        <v>0</v>
+      </c>
+      <c r="J95" s="12" t="n">
+        <f aca="false">I95*$B$8/12</f>
+        <v>0</v>
+      </c>
+      <c r="K95" s="12" t="n">
+        <f aca="false">MIN(I95+J95,J95+$B$9*I95)</f>
+        <v>0</v>
+      </c>
+      <c r="L95" s="12" t="n">
+        <f aca="false">MIN(I95+J95,MAX(D95-G95,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M95" s="12" t="n">
+        <f aca="false">I95+J95-L95</f>
+        <v>0</v>
+      </c>
+      <c r="N95" s="12" t="n">
+        <f aca="false">P94</f>
+        <v>84581.25</v>
+      </c>
+      <c r="O95" s="12" t="n">
+        <f aca="false">MIN(D95-G95-L95,MAX($B$15-$B$18-N95,0))</f>
+        <v>0</v>
+      </c>
+      <c r="P95" s="12" t="n">
+        <f aca="false">N95+O95</f>
+        <v>84581.25</v>
+      </c>
+      <c r="Q95" s="5" t="n">
+        <f aca="false">IF(H95&lt;=0.005,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="R95" s="5" t="n">
+        <f aca="false">IF(M95&lt;=0.005,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="S95" s="5" t="n">
+        <f aca="false">IF(AND(Q95=1,R95=1),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="T95" s="5" t="n">
+        <f aca="false">IF(P95&gt;=$B$20,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="U95" s="5" t="n">
+        <f aca="false">IF(P95+$B$18&gt;=$B$15-0.5,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="V95" s="12" t="n">
+        <f aca="false">MAX(D95-G95-L95,0)-MAX(O95,0)</f>
+        <v>2911.09333333334</v>
+      </c>
+      <c r="W95" s="12" t="n">
+        <f aca="false">P95+$B$18</f>
         <v>100842</v>
       </c>
     </row>
@@ -9702,12 +9753,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9715,48 +9766,48 @@
         <v>13</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="M4" s="10" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="N4" s="10" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -9774,7 +9825,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="B6" s="13" t="n">
         <v>17767.46</v>
@@ -9821,7 +9872,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="B7" s="13" t="n">
         <v>6410.38</v>
@@ -9868,7 +9919,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="B8" s="13" t="n">
         <v>1459.54</v>
@@ -9915,7 +9966,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="B9" s="17" t="n">
         <f aca="false">SUM(B6:B8)</f>
@@ -9972,7 +10023,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -9990,7 +10041,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="B12" s="13" t="n">
         <v>4300</v>
@@ -10037,7 +10088,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="B13" s="13" t="n">
         <v>32.71</v>
@@ -10084,7 +10135,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="B14" s="13" t="n">
         <v>0</v>
@@ -10131,7 +10182,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="B15" s="13" t="n">
         <v>183.82</v>
@@ -10178,7 +10229,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="B16" s="13" t="n">
         <v>500</v>
@@ -10225,7 +10276,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="B17" s="17" t="n">
         <f aca="false">SUM(B12:B16)</f>
@@ -10282,7 +10333,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -10300,7 +10351,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
       <c r="B20" s="13" t="n">
         <v>6857.93</v>
@@ -10394,7 +10445,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="B22" s="13" t="n">
         <v>1057.39</v>
@@ -10441,7 +10492,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="B23" s="13" t="n">
         <v>341.99</v>
@@ -10488,7 +10539,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="B24" s="13" t="n">
         <v>0</v>
@@ -10535,7 +10586,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="B25" s="13" t="n">
         <v>856.83</v>
@@ -10582,7 +10633,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
       <c r="B26" s="13" t="n">
         <v>286.67</v>
@@ -10629,7 +10680,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="B27" s="13" t="n">
         <v>614</v>
@@ -10676,7 +10727,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="B28" s="13" t="n">
         <v>323.39</v>
@@ -10723,7 +10774,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="B29" s="13" t="n">
         <v>368.15</v>
@@ -10770,7 +10821,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="B30" s="13" t="n">
         <v>400.62</v>
@@ -10817,7 +10868,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="B31" s="13" t="n">
         <v>134.97</v>
@@ -10864,7 +10915,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="B32" s="13" t="n">
         <v>178.9</v>
@@ -10911,7 +10962,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="B33" s="13" t="n">
         <v>115.5</v>
@@ -10958,7 +11009,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="B34" s="13" t="n">
         <v>760</v>
@@ -11005,7 +11056,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="B35" s="13" t="n">
         <v>155</v>
@@ -11099,7 +11150,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="B37" s="13" t="n">
         <v>473.56</v>
@@ -11146,7 +11197,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="B38" s="13" t="n">
         <v>431.52</v>
@@ -11193,7 +11244,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="B39" s="13" t="n">
         <v>359.9</v>
@@ -11240,7 +11291,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="B40" s="13" t="n">
         <v>27.6</v>
@@ -11287,7 +11338,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="B41" s="13" t="n">
         <v>557.68</v>
@@ -11334,7 +11385,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="B42" s="13" t="n">
         <v>385.13</v>
@@ -11381,7 +11432,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="B43" s="13" t="n">
         <v>209</v>
@@ -11428,7 +11479,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="B44" s="13" t="n">
         <v>266.15</v>
@@ -11522,7 +11573,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="B46" s="13" t="n">
         <v>469.36</v>
@@ -11616,7 +11667,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="B48" s="13" t="n">
         <v>72.9</v>
@@ -11663,7 +11714,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="B49" s="13" t="n">
         <v>0.5</v>
@@ -11710,7 +11761,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="B50" s="13" t="n">
         <v>355.78</v>
@@ -11757,7 +11808,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="B51" s="13" t="n">
         <v>97.3</v>
@@ -11804,7 +11855,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="B52" s="13" t="n">
         <v>129.41</v>
@@ -11851,7 +11902,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="B53" s="13" t="n">
         <v>465.78</v>
@@ -11898,7 +11949,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="B54" s="13" t="n">
         <v>240</v>
@@ -11945,7 +11996,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="B55" s="13" t="n">
         <v>729.5</v>
@@ -11992,7 +12043,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="B56" s="13" t="n">
         <v>2.25</v>
@@ -12039,7 +12090,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="B57" s="13" t="n">
         <v>0</v>
@@ -12086,7 +12137,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="B58" s="13" t="n">
         <v>127.73</v>
@@ -12133,7 +12184,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="15" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="B59" s="17" t="n">
         <f aca="false">SUM(B20:B58)</f>
@@ -12190,7 +12241,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="8" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="B61" s="28" t="n">
         <f aca="false">B17+B59</f>
@@ -12247,7 +12298,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="8" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="B62" s="28" t="n">
         <f aca="false">B9</f>
@@ -12304,7 +12355,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="8" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="B63" s="9" t="n">
         <f aca="false">B62-B61</f>
@@ -12390,35 +12441,35 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="H4" s="10" t="s">
         <v>20</v>
@@ -12426,10 +12477,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>72.97</v>
@@ -12439,25 +12490,25 @@
         <v>875.64</v>
       </c>
       <c r="E5" s="35" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="F5" s="12" t="n">
         <f aca="false">IF(E5="Cut",D5,0)</f>
         <v>0</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>82.99</v>
@@ -12467,25 +12518,25 @@
         <v>995.88</v>
       </c>
       <c r="E6" s="35" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F6" s="12" t="n">
         <f aca="false">IF(E6="Cut",D6,0)</f>
         <v>0</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>26.99</v>
@@ -12495,23 +12546,23 @@
         <v>323.88</v>
       </c>
       <c r="E7" s="35" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="F7" s="12" t="n">
         <f aca="false">IF(E7="Cut",D7,0)</f>
         <v>0</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="H7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>18.99</v>
@@ -12521,25 +12572,25 @@
         <v>227.88</v>
       </c>
       <c r="E8" s="35" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F8" s="12" t="n">
         <f aca="false">IF(E8="Cut",D8,0)</f>
         <v>0</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>12.99</v>
@@ -12549,23 +12600,23 @@
         <v>155.88</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="F9" s="12" t="n">
         <f aca="false">IF(E9="Cut",D9,0)</f>
         <v>0</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="H9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>139</v>
@@ -12575,25 +12626,25 @@
         <v>139</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="F10" s="12" t="n">
         <f aca="false">IF(E10="Cut",D10,0)</f>
         <v>0</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C11" s="6" t="n">
         <v>4.99</v>
@@ -12603,25 +12654,25 @@
         <v>59.88</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F11" s="12" t="n">
         <f aca="false">IF(E11="Cut",D11,0)</f>
         <v>0</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>6.36</v>
@@ -12631,25 +12682,25 @@
         <v>76.32</v>
       </c>
       <c r="E12" s="35" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F12" s="12" t="n">
         <f aca="false">IF(E12="Cut",D12,0)</f>
         <v>0</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C13" s="6" t="n">
         <v>11.99</v>
@@ -12659,25 +12710,25 @@
         <v>143.88</v>
       </c>
       <c r="E13" s="35" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F13" s="12" t="n">
         <f aca="false">IF(E13="Cut",D13,0)</f>
         <v>0</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C14" s="6" t="n">
         <v>8.99</v>
@@ -12687,25 +12738,25 @@
         <v>107.88</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F14" s="12" t="n">
         <f aca="false">IF(E14="Cut",D14,0)</f>
         <v>0</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C15" s="6" t="n">
         <v>25</v>
@@ -12715,25 +12766,25 @@
         <v>300</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F15" s="12" t="n">
         <f aca="false">IF(E15="Cut",D15,0)</f>
         <v>0</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C16" s="6" t="n">
         <v>27.72</v>
@@ -12743,25 +12794,25 @@
         <v>332.64</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F16" s="12" t="n">
         <f aca="false">IF(E16="Cut",D16,0)</f>
         <v>0</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="C17" s="6" t="n">
         <v>99.99</v>
@@ -12771,23 +12822,23 @@
         <v>99.99</v>
       </c>
       <c r="E17" s="35" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F17" s="12" t="n">
         <f aca="false">IF(E17="Cut",D17,0)</f>
         <v>0</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="H17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="C18" s="6" t="n">
         <v>150</v>
@@ -12797,23 +12848,23 @@
         <v>150</v>
       </c>
       <c r="E18" s="35" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F18" s="12" t="n">
         <f aca="false">IF(E18="Cut",D18,0)</f>
         <v>0</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
       <c r="H18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C19" s="6" t="n">
         <v>20.7</v>
@@ -12823,25 +12874,25 @@
         <v>248.4</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="F19" s="12" t="n">
         <f aca="false">IF(E19="Cut",D19,0)</f>
         <v>0</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>408</v>
+        <v>414</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>409</v>
+        <v>415</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C20" s="6" t="n">
         <v>10</v>
@@ -12851,25 +12902,25 @@
         <v>120</v>
       </c>
       <c r="E20" s="35" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="F20" s="12" t="n">
         <f aca="false">IF(E20="Cut",D20,0)</f>
         <v>0</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>410</v>
+        <v>416</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>32.99</v>
@@ -12879,25 +12930,25 @@
         <v>395.88</v>
       </c>
       <c r="E21" s="35" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F21" s="12" t="n">
         <f aca="false">IF(E21="Cut",D21,0)</f>
         <v>0</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>412</v>
+        <v>418</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>413</v>
+        <v>419</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C22" s="6" t="n">
         <v>13.94</v>
@@ -12907,25 +12958,25 @@
         <v>167.28</v>
       </c>
       <c r="E22" s="35" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F22" s="12" t="n">
         <f aca="false">IF(E22="Cut",D22,0)</f>
         <v>0</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C23" s="6" t="n">
         <v>20.76</v>
@@ -12935,25 +12986,25 @@
         <v>249.12</v>
       </c>
       <c r="E23" s="35" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F23" s="12" t="n">
         <f aca="false">IF(E23="Cut",D23,0)</f>
         <v>0</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>419</v>
+        <v>425</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>420</v>
+        <v>426</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C24" s="6" t="n">
         <v>10.63</v>
@@ -12963,23 +13014,23 @@
         <v>127.56</v>
       </c>
       <c r="E24" s="35" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="F24" s="12" t="n">
         <f aca="false">IF(E24="Cut",D24,0)</f>
         <v>0</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>421</v>
+        <v>427</v>
       </c>
       <c r="H24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>422</v>
+        <v>428</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C25" s="6" t="n">
         <v>21.25</v>
@@ -12989,23 +13040,23 @@
         <v>255</v>
       </c>
       <c r="E25" s="35" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="F25" s="12" t="n">
         <f aca="false">IF(E25="Cut",D25,0)</f>
         <v>0</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
       <c r="H25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>423</v>
+        <v>429</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="C26" s="6" t="n">
         <v>381.44</v>
@@ -13015,25 +13066,25 @@
         <v>381.44</v>
       </c>
       <c r="E26" s="35" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="F26" s="12" t="n">
         <f aca="false">IF(E26="Cut",D26,0)</f>
         <v>0</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>424</v>
+        <v>430</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>425</v>
+        <v>431</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>426</v>
+        <v>432</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="C27" s="6" t="n">
         <v>212.49</v>
@@ -13043,25 +13094,25 @@
         <v>212.49</v>
       </c>
       <c r="E27" s="35" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F27" s="12" t="n">
         <f aca="false">IF(E27="Cut",D27,0)</f>
         <v>0</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>428</v>
+        <v>434</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>430</v>
+        <v>436</v>
       </c>
       <c r="C28" s="6" t="n">
         <v>114.75</v>
@@ -13071,25 +13122,25 @@
         <v>229.5</v>
       </c>
       <c r="E28" s="35" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F28" s="12" t="n">
         <f aca="false">IF(E28="Cut",D28,0)</f>
         <v>0</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>432</v>
+        <v>438</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="C29" s="6" t="n">
         <v>548</v>
@@ -13099,25 +13150,25 @@
         <v>548</v>
       </c>
       <c r="E29" s="35" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="F29" s="12" t="n">
         <f aca="false">IF(E29="Cut",D29,0)</f>
         <v>0</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>434</v>
+        <v>440</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>435</v>
+        <v>441</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>436</v>
+        <v>442</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C30" s="6" t="n">
         <v>32.95</v>
@@ -13127,25 +13178,25 @@
         <v>395.4</v>
       </c>
       <c r="E30" s="35" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F30" s="12" t="n">
         <f aca="false">IF(E30="Cut",D30,0)</f>
         <v>0</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>438</v>
+        <v>444</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C31" s="6" t="n">
         <v>115.23</v>
@@ -13155,25 +13206,25 @@
         <v>1382.76</v>
       </c>
       <c r="E31" s="35" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="F31" s="12" t="n">
         <f aca="false">IF(E31="Cut",D31,0)</f>
         <v>0</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>441</v>
+        <v>447</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="C32" s="6" t="n">
         <v>25</v>
@@ -13183,22 +13234,22 @@
         <v>300</v>
       </c>
       <c r="E32" s="35" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="F32" s="12" t="n">
         <f aca="false">IF(E32="Cut",D32,0)</f>
         <v>0</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>442</v>
+        <v>448</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
       <c r="D33" s="17" t="n">
         <f aca="false">SUM(D5:D32)</f>
@@ -13211,7 +13262,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="D34" s="12" t="n">
         <f aca="false">SUMIF(E5:E32,"Review",D5:D32)</f>
@@ -13220,7 +13271,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>446</v>
+        <v>452</v>
       </c>
     </row>
   </sheetData>
@@ -13248,156 +13299,156 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="36" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>449</v>
+        <v>455</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="36" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>451</v>
+        <v>457</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="36" t="s">
-        <v>452</v>
+        <v>458</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="36" t="s">
-        <v>454</v>
+        <v>460</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="36" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
       <c r="B7" s="37" t="s">
-        <v>457</v>
+        <v>463</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="36" t="s">
-        <v>458</v>
+        <v>464</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="36" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="36" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="36" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="36" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="B15" s="37" t="s">
-        <v>470</v>
+        <v>476</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="B16" s="37" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="B18" s="37" t="s">
-        <v>473</v>
+        <v>479</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="B19" s="37" t="s">
-        <v>474</v>
+        <v>480</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="B20" s="37" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="B21" s="37" t="s">
-        <v>476</v>
+        <v>482</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="B22" s="37" t="s">
-        <v>477</v>
+        <v>483</v>
       </c>
     </row>
   </sheetData>

</xml_diff>